<commit_message>
feat(tc-studio): integrate import workflows and remove AUTO classification
Add persistent library import previews, explicit conflict decisions, multi-file and per-sheet mapping, profile CRUD, history and rollback. Redirect the retired Import Studio UI while preserving shared engines and legacy data/API compatibility.

User-requested change from the original phase plans: remove AUTO from Studio controls, generation schema, validation, filtering and Markdown eligibility, and remove its Excel column/summary while preserving formulas and original workbooks. Keep historical plans as records; update current docs and blank template.

Verified RED-to-GREEN regressions, 856 unit tests passed (1 skipped), 178 TC library tests passed, and headed Playwright import/edit/conflict/rollback/actual local Claude generation/approval/XLSX and Markdown export. No push.
</commit_message>
<xml_diff>
--- a/doc/guides/tc-studio/templates/TC_빈양식.xlsx
+++ b/doc/guides/tc-studio/templates/TC_빈양식.xlsx
@@ -955,7 +955,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="B1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="14.75" customWidth="1" style="123" min="2" max="2"/>
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q266"/>
+  <dimension ref="A1:P266"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="4.25" customWidth="1" style="123" min="1" max="1"/>
@@ -1059,7 +1059,6 @@
       <c r="N1" s="125" t="n"/>
       <c r="O1" s="8" t="n"/>
       <c r="P1" s="8" t="n"/>
-      <c r="Q1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="9" t="n"/>
@@ -1087,14 +1086,9 @@
         </is>
       </c>
       <c r="M2" s="125" t="n"/>
-      <c r="N2" s="129" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
+      <c r="N2" s="16" t="n"/>
       <c r="O2" s="16" t="n"/>
       <c r="P2" s="16" t="n"/>
-      <c r="Q2" s="16" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n"/>
@@ -1126,10 +1120,9 @@
           <t>iOS</t>
         </is>
       </c>
-      <c r="N3" s="131" t="n"/>
+      <c r="N3" s="16" t="n"/>
       <c r="O3" s="16" t="n"/>
       <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n"/>
@@ -1146,11 +1139,11 @@
         </is>
       </c>
       <c r="J4" s="22">
+        <f>COUNTIF(J13:J18,I4)</f>
+        <v/>
+      </c>
+      <c r="K4" s="22">
         <f>COUNTIF(K13:K18,I4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="22">
-        <f>COUNTIF(L13:L18,I4)</f>
         <v/>
       </c>
       <c r="L4" s="23">
@@ -1161,10 +1154,9 @@
         <f>IFERROR((SUM(K4:K6)/K9),"-")</f>
         <v/>
       </c>
-      <c r="N4" s="131" t="n"/>
+      <c r="N4" s="16" t="n"/>
       <c r="O4" s="16" t="n"/>
       <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="16" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n"/>
@@ -1181,11 +1173,11 @@
         </is>
       </c>
       <c r="J5" s="22">
+        <f>COUNTIF(J18:J20,I5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="22">
         <f>COUNTIF(K18:K20,I5)</f>
-        <v/>
-      </c>
-      <c r="K5" s="22">
-        <f>COUNTIF(L18:L20,I5)</f>
         <v/>
       </c>
       <c r="L5" s="132" t="inlineStr">
@@ -1194,10 +1186,9 @@
         </is>
       </c>
       <c r="M5" s="133" t="n"/>
-      <c r="N5" s="131" t="n"/>
+      <c r="N5" s="16" t="n"/>
       <c r="O5" s="16" t="n"/>
       <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n"/>
@@ -1214,11 +1205,11 @@
         </is>
       </c>
       <c r="J6" s="22">
+        <f>COUNTIF(J20:J37,I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="22">
         <f>COUNTIF(K20:K37,I6)</f>
-        <v/>
-      </c>
-      <c r="K6" s="22">
-        <f>COUNTIF(L20:L37,I6)</f>
         <v/>
       </c>
       <c r="L6" s="19" t="inlineStr">
@@ -1231,10 +1222,9 @@
           <t>iOS</t>
         </is>
       </c>
-      <c r="N6" s="133" t="n"/>
+      <c r="N6" s="16" t="n"/>
       <c r="O6" s="16" t="n"/>
       <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>
@@ -1251,11 +1241,11 @@
         </is>
       </c>
       <c r="J7" s="22">
+        <f>COUNTIF(J37:J78,I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="22">
         <f>COUNTIF(K37:K78,I7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="22">
-        <f>COUNTIF(L37:L78,I7)</f>
         <v/>
       </c>
       <c r="L7" s="23">
@@ -1266,17 +1256,9 @@
         <f>K4/K9</f>
         <v/>
       </c>
-      <c r="N7" s="134">
-        <f>IFERROR(
-  (COUNTIFS(I:I, "P0", J:J, "AUTO") + COUNTIFS(I:I, "P1", J:J, "AUTO")) /
-  (COUNTIF(I:I, "P0") + COUNTIF(I:I, "P1")),
-  0
-)</f>
-        <v/>
-      </c>
+      <c r="N7" s="16" t="n"/>
       <c r="O7" s="16" t="n"/>
       <c r="P7" s="16" t="n"/>
-      <c r="Q7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1309,10 +1291,9 @@
         <f>average(L4:M4)</f>
         <v/>
       </c>
-      <c r="N8" s="131" t="n"/>
+      <c r="N8" s="16" t="n"/>
       <c r="O8" s="16" t="n"/>
       <c r="P8" s="16" t="n"/>
-      <c r="Q8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n"/>
@@ -1344,10 +1325,9 @@
         <f>average(L7:M7)</f>
         <v/>
       </c>
-      <c r="N9" s="133" t="n"/>
+      <c r="N9" s="16" t="n"/>
       <c r="O9" s="16" t="n"/>
       <c r="P9" s="16" t="n"/>
-      <c r="Q9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n"/>
@@ -1361,12 +1341,11 @@
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="8" t="n"/>
+      <c r="L10" s="8" t="n"/>
+      <c r="M10" s="16" t="n"/>
       <c r="N10" s="16" t="n"/>
       <c r="O10" s="16" t="n"/>
       <c r="P10" s="16" t="n"/>
-      <c r="Q10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
@@ -1416,24 +1395,19 @@
       </c>
       <c r="J11" s="42" t="inlineStr">
         <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="K11" s="42" t="inlineStr">
-        <is>
           <t>환경</t>
         </is>
       </c>
-      <c r="L11" s="125" t="n"/>
-      <c r="M11" s="42" t="inlineStr">
+      <c r="K11" s="125" t="n"/>
+      <c r="L11" s="42" t="inlineStr">
         <is>
           <t>기타</t>
         </is>
       </c>
-      <c r="N11" s="135" t="n"/>
+      <c r="M11" s="135" t="n"/>
+      <c r="N11" s="40" t="n"/>
       <c r="O11" s="40" t="n"/>
       <c r="P11" s="40" t="n"/>
-      <c r="Q11" s="40" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="130" t="n"/>
@@ -1445,22 +1419,21 @@
       <c r="G12" s="130" t="n"/>
       <c r="H12" s="130" t="n"/>
       <c r="I12" s="41" t="n"/>
-      <c r="J12" s="130" t="n"/>
-      <c r="K12" s="42" t="inlineStr">
+      <c r="J12" s="42" t="inlineStr">
         <is>
           <t>And</t>
         </is>
       </c>
-      <c r="L12" s="42" t="inlineStr">
+      <c r="K12" s="42" t="inlineStr">
         <is>
           <t>iOS</t>
         </is>
       </c>
-      <c r="M12" s="136" t="n"/>
-      <c r="N12" s="133" t="n"/>
+      <c r="L12" s="136" t="n"/>
+      <c r="M12" s="133" t="n"/>
+      <c r="N12" s="40" t="n"/>
       <c r="O12" s="40" t="n"/>
       <c r="P12" s="40" t="n"/>
-      <c r="Q12" s="40" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="74" t="n"/>
@@ -1472,13 +1445,12 @@
       <c r="G13" s="114" t="n"/>
       <c r="H13" s="114" t="n"/>
       <c r="I13" s="53" t="n"/>
-      <c r="J13" s="55" t="n"/>
+      <c r="J13" s="74" t="n"/>
       <c r="K13" s="74" t="n"/>
-      <c r="L13" s="74" t="n"/>
-      <c r="M13" s="100" t="n"/>
+      <c r="L13" s="100" t="n"/>
+      <c r="N13" s="57" t="n"/>
       <c r="O13" s="57" t="n"/>
       <c r="P13" s="57" t="n"/>
-      <c r="Q13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="74" t="n"/>
@@ -1487,26 +1459,24 @@
       <c r="G14" s="114" t="n"/>
       <c r="H14" s="114" t="n"/>
       <c r="I14" s="53" t="n"/>
-      <c r="J14" s="55" t="n"/>
+      <c r="J14" s="74" t="n"/>
       <c r="K14" s="74" t="n"/>
-      <c r="L14" s="74" t="n"/>
-      <c r="M14" s="100" t="n"/>
+      <c r="L14" s="100" t="n"/>
+      <c r="N14" s="57" t="n"/>
       <c r="O14" s="57" t="n"/>
       <c r="P14" s="57" t="n"/>
-      <c r="Q14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="74" t="n"/>
       <c r="G15" s="114" t="n"/>
       <c r="H15" s="114" t="n"/>
       <c r="I15" s="53" t="n"/>
-      <c r="J15" s="55" t="n"/>
+      <c r="J15" s="74" t="n"/>
       <c r="K15" s="74" t="n"/>
-      <c r="L15" s="74" t="n"/>
-      <c r="M15" s="100" t="n"/>
+      <c r="L15" s="100" t="n"/>
+      <c r="N15" s="57" t="n"/>
       <c r="O15" s="57" t="n"/>
       <c r="P15" s="57" t="n"/>
-      <c r="Q15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="74" t="n"/>
@@ -1514,26 +1484,24 @@
       <c r="G16" s="93" t="n"/>
       <c r="H16" s="93" t="n"/>
       <c r="I16" s="53" t="n"/>
-      <c r="J16" s="55" t="n"/>
+      <c r="J16" s="74" t="n"/>
       <c r="K16" s="74" t="n"/>
-      <c r="L16" s="74" t="n"/>
-      <c r="M16" s="100" t="n"/>
+      <c r="L16" s="100" t="n"/>
+      <c r="N16" s="57" t="n"/>
       <c r="O16" s="57" t="n"/>
       <c r="P16" s="57" t="n"/>
-      <c r="Q16" s="57" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="74" t="n"/>
       <c r="G17" s="93" t="n"/>
       <c r="H17" s="93" t="n"/>
       <c r="I17" s="53" t="n"/>
-      <c r="J17" s="55" t="n"/>
+      <c r="J17" s="74" t="n"/>
       <c r="K17" s="74" t="n"/>
-      <c r="L17" s="74" t="n"/>
-      <c r="M17" s="100" t="n"/>
+      <c r="L17" s="100" t="n"/>
+      <c r="N17" s="57" t="n"/>
       <c r="O17" s="57" t="n"/>
       <c r="P17" s="57" t="n"/>
-      <c r="Q17" s="57" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="74" t="n"/>
@@ -1545,13 +1513,12 @@
       <c r="G18" s="114" t="n"/>
       <c r="H18" s="114" t="n"/>
       <c r="I18" s="53" t="n"/>
-      <c r="J18" s="55" t="n"/>
+      <c r="J18" s="74" t="n"/>
       <c r="K18" s="74" t="n"/>
-      <c r="L18" s="74" t="n"/>
-      <c r="M18" s="100" t="n"/>
+      <c r="L18" s="100" t="n"/>
+      <c r="N18" s="57" t="n"/>
       <c r="O18" s="57" t="n"/>
       <c r="P18" s="57" t="n"/>
-      <c r="Q18" s="57" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="74" t="n"/>
@@ -1560,26 +1527,24 @@
       <c r="G19" s="114" t="n"/>
       <c r="H19" s="114" t="n"/>
       <c r="I19" s="53" t="n"/>
-      <c r="J19" s="55" t="n"/>
+      <c r="J19" s="74" t="n"/>
       <c r="K19" s="74" t="n"/>
-      <c r="L19" s="74" t="n"/>
-      <c r="M19" s="100" t="n"/>
+      <c r="L19" s="100" t="n"/>
+      <c r="N19" s="57" t="n"/>
       <c r="O19" s="57" t="n"/>
       <c r="P19" s="57" t="n"/>
-      <c r="Q19" s="57" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="74" t="n"/>
       <c r="G20" s="114" t="n"/>
       <c r="H20" s="114" t="n"/>
       <c r="I20" s="53" t="n"/>
-      <c r="J20" s="55" t="n"/>
+      <c r="J20" s="74" t="n"/>
       <c r="K20" s="74" t="n"/>
-      <c r="L20" s="74" t="n"/>
-      <c r="M20" s="100" t="n"/>
+      <c r="L20" s="100" t="n"/>
+      <c r="N20" s="57" t="n"/>
       <c r="O20" s="57" t="n"/>
       <c r="P20" s="57" t="n"/>
-      <c r="Q20" s="57" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="74" t="n"/>
@@ -1587,13 +1552,12 @@
       <c r="G21" s="114" t="n"/>
       <c r="H21" s="114" t="n"/>
       <c r="I21" s="53" t="n"/>
-      <c r="J21" s="55" t="n"/>
+      <c r="J21" s="74" t="n"/>
       <c r="K21" s="74" t="n"/>
-      <c r="L21" s="74" t="n"/>
-      <c r="M21" s="100" t="n"/>
+      <c r="L21" s="100" t="n"/>
+      <c r="N21" s="57" t="n"/>
       <c r="O21" s="57" t="n"/>
       <c r="P21" s="57" t="n"/>
-      <c r="Q21" s="57" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="74" t="n"/>
@@ -1601,13 +1565,12 @@
       <c r="G22" s="114" t="n"/>
       <c r="H22" s="114" t="n"/>
       <c r="I22" s="53" t="n"/>
-      <c r="J22" s="55" t="n"/>
+      <c r="J22" s="74" t="n"/>
       <c r="K22" s="74" t="n"/>
-      <c r="L22" s="74" t="n"/>
-      <c r="M22" s="100" t="n"/>
+      <c r="L22" s="100" t="n"/>
+      <c r="N22" s="57" t="n"/>
       <c r="O22" s="57" t="n"/>
       <c r="P22" s="57" t="n"/>
-      <c r="Q22" s="57" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="74" t="n"/>
@@ -1618,39 +1581,36 @@
       <c r="G23" s="114" t="n"/>
       <c r="H23" s="114" t="n"/>
       <c r="I23" s="53" t="n"/>
-      <c r="J23" s="55" t="n"/>
+      <c r="J23" s="74" t="n"/>
       <c r="K23" s="74" t="n"/>
-      <c r="L23" s="74" t="n"/>
-      <c r="M23" s="100" t="n"/>
+      <c r="L23" s="100" t="n"/>
+      <c r="N23" s="57" t="n"/>
       <c r="O23" s="57" t="n"/>
       <c r="P23" s="57" t="n"/>
-      <c r="Q23" s="57" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="74" t="n"/>
       <c r="G24" s="114" t="n"/>
       <c r="H24" s="114" t="n"/>
       <c r="I24" s="53" t="n"/>
-      <c r="J24" s="55" t="n"/>
+      <c r="J24" s="74" t="n"/>
       <c r="K24" s="74" t="n"/>
-      <c r="L24" s="74" t="n"/>
-      <c r="M24" s="100" t="n"/>
+      <c r="L24" s="100" t="n"/>
+      <c r="N24" s="57" t="n"/>
       <c r="O24" s="57" t="n"/>
       <c r="P24" s="57" t="n"/>
-      <c r="Q24" s="57" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="74" t="n"/>
       <c r="G25" s="114" t="n"/>
       <c r="H25" s="114" t="n"/>
       <c r="I25" s="53" t="n"/>
-      <c r="J25" s="55" t="n"/>
+      <c r="J25" s="74" t="n"/>
       <c r="K25" s="74" t="n"/>
-      <c r="L25" s="74" t="n"/>
-      <c r="M25" s="100" t="n"/>
+      <c r="L25" s="100" t="n"/>
+      <c r="N25" s="57" t="n"/>
       <c r="O25" s="57" t="n"/>
       <c r="P25" s="57" t="n"/>
-      <c r="Q25" s="57" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="74" t="n"/>
@@ -1660,13 +1620,12 @@
       <c r="G26" s="114" t="n"/>
       <c r="H26" s="114" t="n"/>
       <c r="I26" s="53" t="n"/>
-      <c r="J26" s="55" t="n"/>
+      <c r="J26" s="74" t="n"/>
       <c r="K26" s="74" t="n"/>
-      <c r="L26" s="74" t="n"/>
-      <c r="M26" s="100" t="n"/>
+      <c r="L26" s="100" t="n"/>
+      <c r="N26" s="57" t="n"/>
       <c r="O26" s="57" t="n"/>
       <c r="P26" s="57" t="n"/>
-      <c r="Q26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="74" t="n"/>
@@ -1674,26 +1633,24 @@
       <c r="G27" s="114" t="n"/>
       <c r="H27" s="114" t="n"/>
       <c r="I27" s="53" t="n"/>
-      <c r="J27" s="55" t="n"/>
+      <c r="J27" s="74" t="n"/>
       <c r="K27" s="74" t="n"/>
-      <c r="L27" s="74" t="n"/>
-      <c r="M27" s="100" t="n"/>
+      <c r="L27" s="100" t="n"/>
+      <c r="N27" s="57" t="n"/>
       <c r="O27" s="57" t="n"/>
       <c r="P27" s="57" t="n"/>
-      <c r="Q27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="74" t="n"/>
       <c r="G28" s="114" t="n"/>
       <c r="H28" s="114" t="n"/>
       <c r="I28" s="53" t="n"/>
-      <c r="J28" s="55" t="n"/>
+      <c r="J28" s="74" t="n"/>
       <c r="K28" s="74" t="n"/>
-      <c r="L28" s="74" t="n"/>
-      <c r="M28" s="100" t="n"/>
+      <c r="L28" s="100" t="n"/>
+      <c r="N28" s="57" t="n"/>
       <c r="O28" s="57" t="n"/>
       <c r="P28" s="57" t="n"/>
-      <c r="Q28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="74" t="n"/>
@@ -1701,13 +1658,12 @@
       <c r="G29" s="114" t="n"/>
       <c r="H29" s="93" t="n"/>
       <c r="I29" s="53" t="n"/>
-      <c r="J29" s="55" t="n"/>
+      <c r="J29" s="74" t="n"/>
       <c r="K29" s="74" t="n"/>
-      <c r="L29" s="74" t="n"/>
-      <c r="M29" s="100" t="n"/>
+      <c r="L29" s="100" t="n"/>
+      <c r="N29" s="57" t="n"/>
       <c r="O29" s="57" t="n"/>
       <c r="P29" s="57" t="n"/>
-      <c r="Q29" s="57" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="74" t="n"/>
@@ -1715,26 +1671,24 @@
       <c r="G30" s="114" t="n"/>
       <c r="H30" s="114" t="n"/>
       <c r="I30" s="53" t="n"/>
-      <c r="J30" s="55" t="n"/>
+      <c r="J30" s="74" t="n"/>
       <c r="K30" s="74" t="n"/>
-      <c r="L30" s="74" t="n"/>
-      <c r="M30" s="100" t="n"/>
+      <c r="L30" s="100" t="n"/>
+      <c r="N30" s="57" t="n"/>
       <c r="O30" s="57" t="n"/>
       <c r="P30" s="57" t="n"/>
-      <c r="Q30" s="57" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="74" t="n"/>
       <c r="G31" s="114" t="n"/>
       <c r="H31" s="114" t="n"/>
       <c r="I31" s="53" t="n"/>
-      <c r="J31" s="55" t="n"/>
+      <c r="J31" s="74" t="n"/>
       <c r="K31" s="74" t="n"/>
-      <c r="L31" s="74" t="n"/>
-      <c r="M31" s="100" t="n"/>
+      <c r="L31" s="100" t="n"/>
+      <c r="N31" s="57" t="n"/>
       <c r="O31" s="57" t="n"/>
       <c r="P31" s="57" t="n"/>
-      <c r="Q31" s="57" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="74" t="n"/>
@@ -1742,13 +1696,12 @@
       <c r="G32" s="114" t="n"/>
       <c r="H32" s="114" t="n"/>
       <c r="I32" s="53" t="n"/>
-      <c r="J32" s="55" t="n"/>
+      <c r="J32" s="74" t="n"/>
       <c r="K32" s="74" t="n"/>
-      <c r="L32" s="74" t="n"/>
-      <c r="M32" s="100" t="n"/>
+      <c r="L32" s="100" t="n"/>
+      <c r="N32" s="57" t="n"/>
       <c r="O32" s="57" t="n"/>
       <c r="P32" s="57" t="n"/>
-      <c r="Q32" s="57" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="74" t="n"/>
@@ -1756,13 +1709,12 @@
       <c r="G33" s="114" t="n"/>
       <c r="H33" s="114" t="n"/>
       <c r="I33" s="53" t="n"/>
-      <c r="J33" s="55" t="n"/>
+      <c r="J33" s="74" t="n"/>
       <c r="K33" s="74" t="n"/>
-      <c r="L33" s="74" t="n"/>
-      <c r="M33" s="100" t="n"/>
+      <c r="L33" s="100" t="n"/>
+      <c r="N33" s="57" t="n"/>
       <c r="O33" s="57" t="n"/>
       <c r="P33" s="57" t="n"/>
-      <c r="Q33" s="57" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="74" t="n"/>
@@ -1770,13 +1722,12 @@
       <c r="G34" s="114" t="n"/>
       <c r="H34" s="114" t="n"/>
       <c r="I34" s="53" t="n"/>
-      <c r="J34" s="55" t="n"/>
+      <c r="J34" s="74" t="n"/>
       <c r="K34" s="74" t="n"/>
-      <c r="L34" s="74" t="n"/>
-      <c r="M34" s="100" t="n"/>
+      <c r="L34" s="100" t="n"/>
+      <c r="N34" s="57" t="n"/>
       <c r="O34" s="57" t="n"/>
       <c r="P34" s="57" t="n"/>
-      <c r="Q34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="74" t="n"/>
@@ -1784,13 +1735,12 @@
       <c r="G35" s="114" t="n"/>
       <c r="H35" s="114" t="n"/>
       <c r="I35" s="53" t="n"/>
-      <c r="J35" s="55" t="n"/>
+      <c r="J35" s="74" t="n"/>
       <c r="K35" s="74" t="n"/>
-      <c r="L35" s="74" t="n"/>
-      <c r="M35" s="100" t="n"/>
+      <c r="L35" s="100" t="n"/>
+      <c r="N35" s="57" t="n"/>
       <c r="O35" s="57" t="n"/>
       <c r="P35" s="57" t="n"/>
-      <c r="Q35" s="57" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="74" t="n"/>
@@ -1801,13 +1751,12 @@
       <c r="G36" s="114" t="n"/>
       <c r="H36" s="114" t="n"/>
       <c r="I36" s="53" t="n"/>
-      <c r="J36" s="55" t="n"/>
+      <c r="J36" s="74" t="n"/>
       <c r="K36" s="74" t="n"/>
-      <c r="L36" s="74" t="n"/>
-      <c r="M36" s="100" t="n"/>
+      <c r="L36" s="100" t="n"/>
+      <c r="N36" s="57" t="n"/>
       <c r="O36" s="57" t="n"/>
       <c r="P36" s="57" t="n"/>
-      <c r="Q36" s="57" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="74" t="n"/>
@@ -1815,13 +1764,12 @@
       <c r="G37" s="114" t="n"/>
       <c r="H37" s="114" t="n"/>
       <c r="I37" s="53" t="n"/>
-      <c r="J37" s="55" t="n"/>
+      <c r="J37" s="74" t="n"/>
       <c r="K37" s="74" t="n"/>
-      <c r="L37" s="74" t="n"/>
-      <c r="M37" s="100" t="n"/>
+      <c r="L37" s="100" t="n"/>
+      <c r="N37" s="57" t="n"/>
       <c r="O37" s="57" t="n"/>
       <c r="P37" s="57" t="n"/>
-      <c r="Q37" s="57" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="74" t="n"/>
@@ -1829,13 +1777,12 @@
       <c r="G38" s="114" t="n"/>
       <c r="H38" s="114" t="n"/>
       <c r="I38" s="53" t="n"/>
-      <c r="J38" s="55" t="n"/>
+      <c r="J38" s="74" t="n"/>
       <c r="K38" s="74" t="n"/>
-      <c r="L38" s="74" t="n"/>
-      <c r="M38" s="100" t="n"/>
+      <c r="L38" s="100" t="n"/>
+      <c r="N38" s="57" t="n"/>
       <c r="O38" s="57" t="n"/>
       <c r="P38" s="57" t="n"/>
-      <c r="Q38" s="57" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="74" t="n"/>
@@ -1843,13 +1790,12 @@
       <c r="G39" s="114" t="n"/>
       <c r="H39" s="114" t="n"/>
       <c r="I39" s="53" t="n"/>
-      <c r="J39" s="55" t="n"/>
+      <c r="J39" s="74" t="n"/>
       <c r="K39" s="74" t="n"/>
-      <c r="L39" s="74" t="n"/>
-      <c r="M39" s="100" t="n"/>
+      <c r="L39" s="100" t="n"/>
+      <c r="N39" s="57" t="n"/>
       <c r="O39" s="57" t="n"/>
       <c r="P39" s="57" t="n"/>
-      <c r="Q39" s="57" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="74" t="n"/>
@@ -1857,13 +1803,12 @@
       <c r="G40" s="114" t="n"/>
       <c r="H40" s="114" t="n"/>
       <c r="I40" s="53" t="n"/>
-      <c r="J40" s="55" t="n"/>
+      <c r="J40" s="74" t="n"/>
       <c r="K40" s="74" t="n"/>
-      <c r="L40" s="74" t="n"/>
-      <c r="M40" s="100" t="n"/>
+      <c r="L40" s="100" t="n"/>
+      <c r="N40" s="57" t="n"/>
       <c r="O40" s="57" t="n"/>
       <c r="P40" s="57" t="n"/>
-      <c r="Q40" s="57" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="74" t="n"/>
@@ -1874,39 +1819,36 @@
       <c r="G41" s="114" t="n"/>
       <c r="H41" s="114" t="n"/>
       <c r="I41" s="53" t="n"/>
-      <c r="J41" s="55" t="n"/>
+      <c r="J41" s="74" t="n"/>
       <c r="K41" s="74" t="n"/>
-      <c r="L41" s="74" t="n"/>
-      <c r="M41" s="100" t="n"/>
+      <c r="L41" s="100" t="n"/>
+      <c r="N41" s="57" t="n"/>
       <c r="O41" s="57" t="n"/>
       <c r="P41" s="57" t="n"/>
-      <c r="Q41" s="57" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="74" t="n"/>
       <c r="G42" s="114" t="n"/>
       <c r="H42" s="114" t="n"/>
       <c r="I42" s="53" t="n"/>
-      <c r="J42" s="55" t="n"/>
+      <c r="J42" s="74" t="n"/>
       <c r="K42" s="74" t="n"/>
-      <c r="L42" s="74" t="n"/>
-      <c r="M42" s="100" t="n"/>
+      <c r="L42" s="100" t="n"/>
+      <c r="N42" s="57" t="n"/>
       <c r="O42" s="57" t="n"/>
       <c r="P42" s="57" t="n"/>
-      <c r="Q42" s="57" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="74" t="n"/>
       <c r="G43" s="114" t="n"/>
       <c r="H43" s="114" t="n"/>
       <c r="I43" s="53" t="n"/>
-      <c r="J43" s="55" t="n"/>
+      <c r="J43" s="74" t="n"/>
       <c r="K43" s="74" t="n"/>
-      <c r="L43" s="74" t="n"/>
-      <c r="M43" s="100" t="n"/>
+      <c r="L43" s="100" t="n"/>
+      <c r="N43" s="57" t="n"/>
       <c r="O43" s="57" t="n"/>
       <c r="P43" s="57" t="n"/>
-      <c r="Q43" s="57" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="74" t="n"/>
@@ -1916,13 +1858,12 @@
       <c r="G44" s="114" t="n"/>
       <c r="H44" s="114" t="n"/>
       <c r="I44" s="53" t="n"/>
-      <c r="J44" s="55" t="n"/>
+      <c r="J44" s="74" t="n"/>
       <c r="K44" s="74" t="n"/>
-      <c r="L44" s="74" t="n"/>
-      <c r="M44" s="100" t="n"/>
+      <c r="L44" s="100" t="n"/>
+      <c r="N44" s="57" t="n"/>
       <c r="O44" s="57" t="n"/>
       <c r="P44" s="57" t="n"/>
-      <c r="Q44" s="57" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="74" t="n"/>
@@ -1930,26 +1871,24 @@
       <c r="G45" s="114" t="n"/>
       <c r="H45" s="114" t="n"/>
       <c r="I45" s="53" t="n"/>
-      <c r="J45" s="55" t="n"/>
+      <c r="J45" s="74" t="n"/>
       <c r="K45" s="74" t="n"/>
-      <c r="L45" s="74" t="n"/>
-      <c r="M45" s="100" t="n"/>
+      <c r="L45" s="100" t="n"/>
+      <c r="N45" s="57" t="n"/>
       <c r="O45" s="57" t="n"/>
       <c r="P45" s="57" t="n"/>
-      <c r="Q45" s="57" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="74" t="n"/>
       <c r="G46" s="114" t="n"/>
       <c r="H46" s="114" t="n"/>
       <c r="I46" s="53" t="n"/>
-      <c r="J46" s="55" t="n"/>
+      <c r="J46" s="74" t="n"/>
       <c r="K46" s="74" t="n"/>
-      <c r="L46" s="74" t="n"/>
-      <c r="M46" s="100" t="n"/>
+      <c r="L46" s="100" t="n"/>
+      <c r="N46" s="57" t="n"/>
       <c r="O46" s="57" t="n"/>
       <c r="P46" s="57" t="n"/>
-      <c r="Q46" s="57" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="74" t="n"/>
@@ -1957,13 +1896,12 @@
       <c r="G47" s="114" t="n"/>
       <c r="H47" s="93" t="n"/>
       <c r="I47" s="53" t="n"/>
-      <c r="J47" s="55" t="n"/>
+      <c r="J47" s="74" t="n"/>
       <c r="K47" s="74" t="n"/>
-      <c r="L47" s="74" t="n"/>
-      <c r="M47" s="100" t="n"/>
+      <c r="L47" s="100" t="n"/>
+      <c r="N47" s="57" t="n"/>
       <c r="O47" s="57" t="n"/>
       <c r="P47" s="57" t="n"/>
-      <c r="Q47" s="57" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="74" t="n"/>
@@ -1971,26 +1909,24 @@
       <c r="G48" s="114" t="n"/>
       <c r="H48" s="114" t="n"/>
       <c r="I48" s="53" t="n"/>
-      <c r="J48" s="55" t="n"/>
+      <c r="J48" s="74" t="n"/>
       <c r="K48" s="74" t="n"/>
-      <c r="L48" s="74" t="n"/>
-      <c r="M48" s="100" t="n"/>
+      <c r="L48" s="100" t="n"/>
+      <c r="N48" s="57" t="n"/>
       <c r="O48" s="57" t="n"/>
       <c r="P48" s="57" t="n"/>
-      <c r="Q48" s="57" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="74" t="n"/>
       <c r="G49" s="114" t="n"/>
       <c r="H49" s="114" t="n"/>
       <c r="I49" s="53" t="n"/>
-      <c r="J49" s="55" t="n"/>
+      <c r="J49" s="74" t="n"/>
       <c r="K49" s="74" t="n"/>
-      <c r="L49" s="74" t="n"/>
-      <c r="M49" s="100" t="n"/>
+      <c r="L49" s="100" t="n"/>
+      <c r="N49" s="57" t="n"/>
       <c r="O49" s="57" t="n"/>
       <c r="P49" s="57" t="n"/>
-      <c r="Q49" s="57" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="74" t="n"/>
@@ -1998,13 +1934,12 @@
       <c r="G50" s="114" t="n"/>
       <c r="H50" s="114" t="n"/>
       <c r="I50" s="53" t="n"/>
-      <c r="J50" s="55" t="n"/>
+      <c r="J50" s="74" t="n"/>
       <c r="K50" s="74" t="n"/>
-      <c r="L50" s="74" t="n"/>
-      <c r="M50" s="100" t="n"/>
+      <c r="L50" s="100" t="n"/>
+      <c r="N50" s="57" t="n"/>
       <c r="O50" s="57" t="n"/>
       <c r="P50" s="57" t="n"/>
-      <c r="Q50" s="57" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="74" t="n"/>
@@ -2012,13 +1947,12 @@
       <c r="G51" s="114" t="n"/>
       <c r="H51" s="114" t="n"/>
       <c r="I51" s="53" t="n"/>
-      <c r="J51" s="55" t="n"/>
+      <c r="J51" s="74" t="n"/>
       <c r="K51" s="74" t="n"/>
-      <c r="L51" s="74" t="n"/>
-      <c r="M51" s="100" t="n"/>
+      <c r="L51" s="100" t="n"/>
+      <c r="N51" s="57" t="n"/>
       <c r="O51" s="57" t="n"/>
       <c r="P51" s="57" t="n"/>
-      <c r="Q51" s="57" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="74" t="n"/>
@@ -2026,13 +1960,12 @@
       <c r="G52" s="114" t="n"/>
       <c r="H52" s="114" t="n"/>
       <c r="I52" s="53" t="n"/>
-      <c r="J52" s="55" t="n"/>
+      <c r="J52" s="74" t="n"/>
       <c r="K52" s="74" t="n"/>
-      <c r="L52" s="74" t="n"/>
-      <c r="M52" s="100" t="n"/>
+      <c r="L52" s="100" t="n"/>
+      <c r="N52" s="57" t="n"/>
       <c r="O52" s="57" t="n"/>
       <c r="P52" s="57" t="n"/>
-      <c r="Q52" s="57" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="74" t="n"/>
@@ -2040,13 +1973,12 @@
       <c r="G53" s="114" t="n"/>
       <c r="H53" s="114" t="n"/>
       <c r="I53" s="53" t="n"/>
-      <c r="J53" s="55" t="n"/>
+      <c r="J53" s="74" t="n"/>
       <c r="K53" s="74" t="n"/>
-      <c r="L53" s="74" t="n"/>
-      <c r="M53" s="100" t="n"/>
+      <c r="L53" s="100" t="n"/>
+      <c r="N53" s="57" t="n"/>
       <c r="O53" s="57" t="n"/>
       <c r="P53" s="57" t="n"/>
-      <c r="Q53" s="57" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="74" t="n"/>
@@ -2057,26 +1989,24 @@
       <c r="G54" s="114" t="n"/>
       <c r="H54" s="50" t="n"/>
       <c r="I54" s="53" t="n"/>
-      <c r="J54" s="55" t="n"/>
+      <c r="J54" s="74" t="n"/>
       <c r="K54" s="74" t="n"/>
-      <c r="L54" s="74" t="n"/>
-      <c r="M54" s="100" t="n"/>
+      <c r="L54" s="100" t="n"/>
+      <c r="N54" s="57" t="n"/>
       <c r="O54" s="57" t="n"/>
       <c r="P54" s="57" t="n"/>
-      <c r="Q54" s="57" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="74" t="n"/>
       <c r="G55" s="114" t="n"/>
       <c r="H55" s="114" t="n"/>
       <c r="I55" s="53" t="n"/>
-      <c r="J55" s="55" t="n"/>
+      <c r="J55" s="74" t="n"/>
       <c r="K55" s="74" t="n"/>
-      <c r="L55" s="74" t="n"/>
-      <c r="M55" s="100" t="n"/>
+      <c r="L55" s="100" t="n"/>
+      <c r="N55" s="57" t="n"/>
       <c r="O55" s="57" t="n"/>
       <c r="P55" s="57" t="n"/>
-      <c r="Q55" s="57" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="74" t="n"/>
@@ -2084,13 +2014,12 @@
       <c r="G56" s="114" t="n"/>
       <c r="H56" s="114" t="n"/>
       <c r="I56" s="53" t="n"/>
-      <c r="J56" s="55" t="n"/>
+      <c r="J56" s="74" t="n"/>
       <c r="K56" s="74" t="n"/>
-      <c r="L56" s="74" t="n"/>
-      <c r="M56" s="100" t="n"/>
+      <c r="L56" s="100" t="n"/>
+      <c r="N56" s="57" t="n"/>
       <c r="O56" s="57" t="n"/>
       <c r="P56" s="57" t="n"/>
-      <c r="Q56" s="57" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="74" t="n"/>
@@ -2098,13 +2027,12 @@
       <c r="G57" s="114" t="n"/>
       <c r="H57" s="114" t="n"/>
       <c r="I57" s="53" t="n"/>
-      <c r="J57" s="55" t="n"/>
+      <c r="J57" s="74" t="n"/>
       <c r="K57" s="74" t="n"/>
-      <c r="L57" s="74" t="n"/>
-      <c r="M57" s="100" t="n"/>
+      <c r="L57" s="100" t="n"/>
+      <c r="N57" s="57" t="n"/>
       <c r="O57" s="57" t="n"/>
       <c r="P57" s="57" t="n"/>
-      <c r="Q57" s="57" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="74" t="n"/>
@@ -2115,13 +2043,12 @@
       <c r="G58" s="93" t="n"/>
       <c r="H58" s="93" t="n"/>
       <c r="I58" s="53" t="n"/>
-      <c r="J58" s="55" t="n"/>
+      <c r="J58" s="74" t="n"/>
       <c r="K58" s="74" t="n"/>
-      <c r="L58" s="74" t="n"/>
-      <c r="M58" s="100" t="n"/>
+      <c r="L58" s="100" t="n"/>
+      <c r="N58" s="57" t="n"/>
       <c r="O58" s="57" t="n"/>
       <c r="P58" s="57" t="n"/>
-      <c r="Q58" s="57" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="74" t="n"/>
@@ -2129,13 +2056,12 @@
       <c r="G59" s="93" t="n"/>
       <c r="H59" s="93" t="n"/>
       <c r="I59" s="53" t="n"/>
-      <c r="J59" s="55" t="n"/>
+      <c r="J59" s="74" t="n"/>
       <c r="K59" s="74" t="n"/>
-      <c r="L59" s="74" t="n"/>
-      <c r="M59" s="100" t="n"/>
+      <c r="L59" s="100" t="n"/>
+      <c r="N59" s="57" t="n"/>
       <c r="O59" s="57" t="n"/>
       <c r="P59" s="57" t="n"/>
-      <c r="Q59" s="57" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="74" t="n"/>
@@ -2143,13 +2069,12 @@
       <c r="G60" s="93" t="n"/>
       <c r="H60" s="93" t="n"/>
       <c r="I60" s="53" t="n"/>
-      <c r="J60" s="55" t="n"/>
+      <c r="J60" s="74" t="n"/>
       <c r="K60" s="74" t="n"/>
-      <c r="L60" s="74" t="n"/>
-      <c r="M60" s="100" t="n"/>
+      <c r="L60" s="100" t="n"/>
+      <c r="N60" s="57" t="n"/>
       <c r="O60" s="57" t="n"/>
       <c r="P60" s="57" t="n"/>
-      <c r="Q60" s="57" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="74" t="n"/>
@@ -2157,13 +2082,12 @@
       <c r="G61" s="93" t="n"/>
       <c r="H61" s="93" t="n"/>
       <c r="I61" s="53" t="n"/>
-      <c r="J61" s="55" t="n"/>
+      <c r="J61" s="74" t="n"/>
       <c r="K61" s="74" t="n"/>
-      <c r="L61" s="74" t="n"/>
-      <c r="M61" s="100" t="n"/>
+      <c r="L61" s="100" t="n"/>
+      <c r="N61" s="57" t="n"/>
       <c r="O61" s="57" t="n"/>
       <c r="P61" s="57" t="n"/>
-      <c r="Q61" s="57" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="74" t="n"/>
@@ -2171,13 +2095,12 @@
       <c r="G62" s="93" t="n"/>
       <c r="H62" s="93" t="n"/>
       <c r="I62" s="53" t="n"/>
-      <c r="J62" s="55" t="n"/>
+      <c r="J62" s="74" t="n"/>
       <c r="K62" s="74" t="n"/>
-      <c r="L62" s="74" t="n"/>
-      <c r="M62" s="100" t="n"/>
+      <c r="L62" s="100" t="n"/>
+      <c r="N62" s="57" t="n"/>
       <c r="O62" s="57" t="n"/>
       <c r="P62" s="57" t="n"/>
-      <c r="Q62" s="57" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="74" t="n"/>
@@ -2185,13 +2108,12 @@
       <c r="G63" s="93" t="n"/>
       <c r="H63" s="93" t="n"/>
       <c r="I63" s="53" t="n"/>
-      <c r="J63" s="55" t="n"/>
+      <c r="J63" s="74" t="n"/>
       <c r="K63" s="74" t="n"/>
-      <c r="L63" s="74" t="n"/>
-      <c r="M63" s="100" t="n"/>
+      <c r="L63" s="100" t="n"/>
+      <c r="N63" s="57" t="n"/>
       <c r="O63" s="57" t="n"/>
       <c r="P63" s="57" t="n"/>
-      <c r="Q63" s="57" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="74" t="n"/>
@@ -2199,13 +2121,12 @@
       <c r="G64" s="93" t="n"/>
       <c r="H64" s="93" t="n"/>
       <c r="I64" s="53" t="n"/>
-      <c r="J64" s="55" t="n"/>
+      <c r="J64" s="74" t="n"/>
       <c r="K64" s="74" t="n"/>
-      <c r="L64" s="74" t="n"/>
-      <c r="M64" s="100" t="n"/>
+      <c r="L64" s="100" t="n"/>
+      <c r="N64" s="57" t="n"/>
       <c r="O64" s="57" t="n"/>
       <c r="P64" s="57" t="n"/>
-      <c r="Q64" s="57" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="74" t="n"/>
@@ -2213,26 +2134,24 @@
       <c r="G65" s="93" t="n"/>
       <c r="H65" s="93" t="n"/>
       <c r="I65" s="53" t="n"/>
-      <c r="J65" s="55" t="n"/>
+      <c r="J65" s="74" t="n"/>
       <c r="K65" s="74" t="n"/>
-      <c r="L65" s="74" t="n"/>
-      <c r="M65" s="100" t="n"/>
+      <c r="L65" s="100" t="n"/>
+      <c r="N65" s="57" t="n"/>
       <c r="O65" s="57" t="n"/>
       <c r="P65" s="57" t="n"/>
-      <c r="Q65" s="57" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="74" t="n"/>
       <c r="G66" s="93" t="n"/>
       <c r="H66" s="93" t="n"/>
       <c r="I66" s="53" t="n"/>
-      <c r="J66" s="55" t="n"/>
+      <c r="J66" s="74" t="n"/>
       <c r="K66" s="74" t="n"/>
-      <c r="L66" s="74" t="n"/>
-      <c r="M66" s="100" t="n"/>
+      <c r="L66" s="100" t="n"/>
+      <c r="N66" s="57" t="n"/>
       <c r="O66" s="57" t="n"/>
       <c r="P66" s="57" t="n"/>
-      <c r="Q66" s="57" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="74" t="n"/>
@@ -2240,26 +2159,24 @@
       <c r="G67" s="93" t="n"/>
       <c r="H67" s="93" t="n"/>
       <c r="I67" s="53" t="n"/>
-      <c r="J67" s="55" t="n"/>
+      <c r="J67" s="74" t="n"/>
       <c r="K67" s="74" t="n"/>
-      <c r="L67" s="74" t="n"/>
-      <c r="M67" s="100" t="n"/>
+      <c r="L67" s="100" t="n"/>
+      <c r="N67" s="57" t="n"/>
       <c r="O67" s="57" t="n"/>
       <c r="P67" s="57" t="n"/>
-      <c r="Q67" s="57" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="74" t="n"/>
       <c r="G68" s="93" t="n"/>
       <c r="H68" s="93" t="n"/>
       <c r="I68" s="53" t="n"/>
-      <c r="J68" s="55" t="n"/>
+      <c r="J68" s="74" t="n"/>
       <c r="K68" s="74" t="n"/>
-      <c r="L68" s="74" t="n"/>
-      <c r="M68" s="100" t="n"/>
+      <c r="L68" s="100" t="n"/>
+      <c r="N68" s="57" t="n"/>
       <c r="O68" s="57" t="n"/>
       <c r="P68" s="57" t="n"/>
-      <c r="Q68" s="57" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="74" t="n"/>
@@ -2267,13 +2184,12 @@
       <c r="G69" s="93" t="n"/>
       <c r="H69" s="93" t="n"/>
       <c r="I69" s="53" t="n"/>
-      <c r="J69" s="55" t="n"/>
+      <c r="J69" s="74" t="n"/>
       <c r="K69" s="74" t="n"/>
-      <c r="L69" s="74" t="n"/>
-      <c r="M69" s="100" t="n"/>
+      <c r="L69" s="100" t="n"/>
+      <c r="N69" s="57" t="n"/>
       <c r="O69" s="57" t="n"/>
       <c r="P69" s="57" t="n"/>
-      <c r="Q69" s="57" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="74" t="n"/>
@@ -2281,13 +2197,12 @@
       <c r="G70" s="93" t="n"/>
       <c r="H70" s="93" t="n"/>
       <c r="I70" s="53" t="n"/>
-      <c r="J70" s="55" t="n"/>
+      <c r="J70" s="74" t="n"/>
       <c r="K70" s="74" t="n"/>
-      <c r="L70" s="74" t="n"/>
-      <c r="M70" s="100" t="n"/>
+      <c r="L70" s="100" t="n"/>
+      <c r="N70" s="57" t="n"/>
       <c r="O70" s="57" t="n"/>
       <c r="P70" s="57" t="n"/>
-      <c r="Q70" s="57" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="74" t="n"/>
@@ -2295,13 +2210,12 @@
       <c r="G71" s="114" t="n"/>
       <c r="H71" s="114" t="n"/>
       <c r="I71" s="53" t="n"/>
-      <c r="J71" s="55" t="n"/>
+      <c r="J71" s="74" t="n"/>
       <c r="K71" s="74" t="n"/>
-      <c r="L71" s="74" t="n"/>
-      <c r="M71" s="100" t="n"/>
+      <c r="L71" s="100" t="n"/>
+      <c r="N71" s="57" t="n"/>
       <c r="O71" s="57" t="n"/>
       <c r="P71" s="57" t="n"/>
-      <c r="Q71" s="57" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="74" t="n"/>
@@ -2309,13 +2223,12 @@
       <c r="G72" s="93" t="n"/>
       <c r="H72" s="93" t="n"/>
       <c r="I72" s="53" t="n"/>
-      <c r="J72" s="55" t="n"/>
+      <c r="J72" s="74" t="n"/>
       <c r="K72" s="74" t="n"/>
-      <c r="L72" s="74" t="n"/>
-      <c r="M72" s="100" t="n"/>
+      <c r="L72" s="100" t="n"/>
+      <c r="N72" s="57" t="n"/>
       <c r="O72" s="57" t="n"/>
       <c r="P72" s="57" t="n"/>
-      <c r="Q72" s="57" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="74" t="n"/>
@@ -2323,13 +2236,12 @@
       <c r="G73" s="93" t="n"/>
       <c r="H73" s="93" t="n"/>
       <c r="I73" s="53" t="n"/>
-      <c r="J73" s="55" t="n"/>
+      <c r="J73" s="74" t="n"/>
       <c r="K73" s="74" t="n"/>
-      <c r="L73" s="74" t="n"/>
-      <c r="M73" s="100" t="n"/>
+      <c r="L73" s="100" t="n"/>
+      <c r="N73" s="57" t="n"/>
       <c r="O73" s="57" t="n"/>
       <c r="P73" s="57" t="n"/>
-      <c r="Q73" s="57" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="74" t="n"/>
@@ -2337,13 +2249,12 @@
       <c r="G74" s="93" t="n"/>
       <c r="H74" s="93" t="n"/>
       <c r="I74" s="53" t="n"/>
-      <c r="J74" s="55" t="n"/>
+      <c r="J74" s="74" t="n"/>
       <c r="K74" s="74" t="n"/>
-      <c r="L74" s="74" t="n"/>
-      <c r="M74" s="100" t="n"/>
+      <c r="L74" s="100" t="n"/>
+      <c r="N74" s="57" t="n"/>
       <c r="O74" s="57" t="n"/>
       <c r="P74" s="57" t="n"/>
-      <c r="Q74" s="57" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="74" t="n"/>
@@ -2354,13 +2265,12 @@
       <c r="G75" s="114" t="n"/>
       <c r="H75" s="50" t="n"/>
       <c r="I75" s="53" t="n"/>
-      <c r="J75" s="55" t="n"/>
+      <c r="J75" s="74" t="n"/>
       <c r="K75" s="74" t="n"/>
-      <c r="L75" s="74" t="n"/>
-      <c r="M75" s="100" t="n"/>
-      <c r="O75" s="92" t="n"/>
+      <c r="L75" s="100" t="n"/>
+      <c r="N75" s="92" t="n"/>
+      <c r="O75" s="57" t="n"/>
       <c r="P75" s="57" t="n"/>
-      <c r="Q75" s="57" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="74" t="n"/>
@@ -2368,13 +2278,12 @@
       <c r="G76" s="114" t="n"/>
       <c r="H76" s="114" t="n"/>
       <c r="I76" s="53" t="n"/>
-      <c r="J76" s="55" t="n"/>
+      <c r="J76" s="74" t="n"/>
       <c r="K76" s="74" t="n"/>
-      <c r="L76" s="74" t="n"/>
-      <c r="M76" s="100" t="n"/>
-      <c r="O76" s="92" t="n"/>
+      <c r="L76" s="100" t="n"/>
+      <c r="N76" s="92" t="n"/>
+      <c r="O76" s="57" t="n"/>
       <c r="P76" s="57" t="n"/>
-      <c r="Q76" s="57" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="74" t="n"/>
@@ -2382,13 +2291,12 @@
       <c r="G77" s="114" t="n"/>
       <c r="H77" s="114" t="n"/>
       <c r="I77" s="53" t="n"/>
-      <c r="J77" s="55" t="n"/>
+      <c r="J77" s="74" t="n"/>
       <c r="K77" s="74" t="n"/>
-      <c r="L77" s="74" t="n"/>
-      <c r="M77" s="100" t="n"/>
-      <c r="O77" s="92" t="n"/>
+      <c r="L77" s="100" t="n"/>
+      <c r="N77" s="92" t="n"/>
+      <c r="O77" s="57" t="n"/>
       <c r="P77" s="57" t="n"/>
-      <c r="Q77" s="57" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="74" t="n"/>
@@ -2396,13 +2304,12 @@
       <c r="G78" s="114" t="n"/>
       <c r="H78" s="114" t="n"/>
       <c r="I78" s="53" t="n"/>
-      <c r="J78" s="55" t="n"/>
+      <c r="J78" s="74" t="n"/>
       <c r="K78" s="74" t="n"/>
-      <c r="L78" s="74" t="n"/>
-      <c r="M78" s="100" t="n"/>
-      <c r="O78" s="92" t="n"/>
+      <c r="L78" s="100" t="n"/>
+      <c r="N78" s="92" t="n"/>
+      <c r="O78" s="57" t="n"/>
       <c r="P78" s="57" t="n"/>
-      <c r="Q78" s="57" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="74" t="n"/>
@@ -2413,13 +2320,12 @@
       <c r="G79" s="114" t="n"/>
       <c r="H79" s="114" t="n"/>
       <c r="I79" s="53" t="n"/>
-      <c r="J79" s="55" t="n"/>
+      <c r="J79" s="74" t="n"/>
       <c r="K79" s="74" t="n"/>
-      <c r="L79" s="74" t="n"/>
-      <c r="M79" s="100" t="n"/>
-      <c r="O79" s="92" t="n"/>
+      <c r="L79" s="100" t="n"/>
+      <c r="N79" s="92" t="n"/>
+      <c r="O79" s="57" t="n"/>
       <c r="P79" s="57" t="n"/>
-      <c r="Q79" s="57" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="74" t="n"/>
@@ -2427,13 +2333,12 @@
       <c r="G80" s="114" t="n"/>
       <c r="H80" s="114" t="n"/>
       <c r="I80" s="53" t="n"/>
-      <c r="J80" s="55" t="n"/>
+      <c r="J80" s="74" t="n"/>
       <c r="K80" s="74" t="n"/>
-      <c r="L80" s="74" t="n"/>
-      <c r="M80" s="100" t="n"/>
-      <c r="O80" s="92" t="n"/>
+      <c r="L80" s="100" t="n"/>
+      <c r="N80" s="92" t="n"/>
+      <c r="O80" s="57" t="n"/>
       <c r="P80" s="57" t="n"/>
-      <c r="Q80" s="57" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="74" t="n"/>
@@ -2441,13 +2346,12 @@
       <c r="G81" s="114" t="n"/>
       <c r="H81" s="114" t="n"/>
       <c r="I81" s="53" t="n"/>
-      <c r="J81" s="55" t="n"/>
+      <c r="J81" s="74" t="n"/>
       <c r="K81" s="74" t="n"/>
-      <c r="L81" s="74" t="n"/>
-      <c r="M81" s="100" t="n"/>
-      <c r="O81" s="92" t="n"/>
+      <c r="L81" s="100" t="n"/>
+      <c r="N81" s="92" t="n"/>
+      <c r="O81" s="57" t="n"/>
       <c r="P81" s="57" t="n"/>
-      <c r="Q81" s="57" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="74" t="n"/>
@@ -2455,13 +2359,12 @@
       <c r="G82" s="114" t="n"/>
       <c r="H82" s="114" t="n"/>
       <c r="I82" s="53" t="n"/>
-      <c r="J82" s="55" t="n"/>
+      <c r="J82" s="74" t="n"/>
       <c r="K82" s="74" t="n"/>
-      <c r="L82" s="74" t="n"/>
-      <c r="M82" s="100" t="n"/>
-      <c r="O82" s="92" t="n"/>
+      <c r="L82" s="100" t="n"/>
+      <c r="N82" s="92" t="n"/>
+      <c r="O82" s="57" t="n"/>
       <c r="P82" s="57" t="n"/>
-      <c r="Q82" s="57" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="74" t="n"/>
@@ -2469,13 +2372,12 @@
       <c r="G83" s="114" t="n"/>
       <c r="H83" s="114" t="n"/>
       <c r="I83" s="53" t="n"/>
-      <c r="J83" s="55" t="n"/>
+      <c r="J83" s="74" t="n"/>
       <c r="K83" s="74" t="n"/>
-      <c r="L83" s="74" t="n"/>
-      <c r="M83" s="100" t="n"/>
-      <c r="O83" s="92" t="n"/>
+      <c r="L83" s="100" t="n"/>
+      <c r="N83" s="92" t="n"/>
+      <c r="O83" s="57" t="n"/>
       <c r="P83" s="57" t="n"/>
-      <c r="Q83" s="57" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="74" t="n"/>
@@ -2483,13 +2385,12 @@
       <c r="G84" s="114" t="n"/>
       <c r="H84" s="114" t="n"/>
       <c r="I84" s="53" t="n"/>
-      <c r="J84" s="55" t="n"/>
+      <c r="J84" s="74" t="n"/>
       <c r="K84" s="74" t="n"/>
-      <c r="L84" s="74" t="n"/>
-      <c r="M84" s="100" t="n"/>
-      <c r="O84" s="92" t="n"/>
+      <c r="L84" s="100" t="n"/>
+      <c r="N84" s="92" t="n"/>
+      <c r="O84" s="57" t="n"/>
       <c r="P84" s="57" t="n"/>
-      <c r="Q84" s="57" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="74" t="n"/>
@@ -2497,13 +2398,12 @@
       <c r="G85" s="114" t="n"/>
       <c r="H85" s="114" t="n"/>
       <c r="I85" s="53" t="n"/>
-      <c r="J85" s="55" t="n"/>
+      <c r="J85" s="74" t="n"/>
       <c r="K85" s="74" t="n"/>
-      <c r="L85" s="74" t="n"/>
-      <c r="M85" s="100" t="n"/>
-      <c r="O85" s="92" t="n"/>
+      <c r="L85" s="100" t="n"/>
+      <c r="N85" s="92" t="n"/>
+      <c r="O85" s="57" t="n"/>
       <c r="P85" s="57" t="n"/>
-      <c r="Q85" s="57" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="74" t="n"/>
@@ -2511,26 +2411,24 @@
       <c r="G86" s="114" t="n"/>
       <c r="H86" s="114" t="n"/>
       <c r="I86" s="53" t="n"/>
-      <c r="J86" s="55" t="n"/>
+      <c r="J86" s="74" t="n"/>
       <c r="K86" s="74" t="n"/>
-      <c r="L86" s="74" t="n"/>
-      <c r="M86" s="100" t="n"/>
-      <c r="O86" s="92" t="n"/>
+      <c r="L86" s="100" t="n"/>
+      <c r="N86" s="92" t="n"/>
+      <c r="O86" s="57" t="n"/>
       <c r="P86" s="57" t="n"/>
-      <c r="Q86" s="57" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="74" t="n"/>
       <c r="G87" s="114" t="n"/>
       <c r="H87" s="114" t="n"/>
       <c r="I87" s="53" t="n"/>
-      <c r="J87" s="55" t="n"/>
+      <c r="J87" s="74" t="n"/>
       <c r="K87" s="74" t="n"/>
-      <c r="L87" s="74" t="n"/>
-      <c r="M87" s="100" t="n"/>
-      <c r="O87" s="92" t="n"/>
+      <c r="L87" s="100" t="n"/>
+      <c r="N87" s="92" t="n"/>
+      <c r="O87" s="57" t="n"/>
       <c r="P87" s="57" t="n"/>
-      <c r="Q87" s="57" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="74" t="n"/>
@@ -2538,26 +2436,24 @@
       <c r="G88" s="114" t="n"/>
       <c r="H88" s="114" t="n"/>
       <c r="I88" s="53" t="n"/>
-      <c r="J88" s="55" t="n"/>
+      <c r="J88" s="74" t="n"/>
       <c r="K88" s="74" t="n"/>
-      <c r="L88" s="74" t="n"/>
-      <c r="M88" s="100" t="n"/>
-      <c r="O88" s="92" t="n"/>
+      <c r="L88" s="100" t="n"/>
+      <c r="N88" s="92" t="n"/>
+      <c r="O88" s="57" t="n"/>
       <c r="P88" s="57" t="n"/>
-      <c r="Q88" s="57" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="74" t="n"/>
       <c r="G89" s="114" t="n"/>
       <c r="H89" s="114" t="n"/>
       <c r="I89" s="53" t="n"/>
-      <c r="J89" s="55" t="n"/>
+      <c r="J89" s="74" t="n"/>
       <c r="K89" s="74" t="n"/>
-      <c r="L89" s="74" t="n"/>
-      <c r="M89" s="100" t="n"/>
-      <c r="O89" s="92" t="n"/>
+      <c r="L89" s="100" t="n"/>
+      <c r="N89" s="92" t="n"/>
+      <c r="O89" s="57" t="n"/>
       <c r="P89" s="57" t="n"/>
-      <c r="Q89" s="57" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="74" t="n"/>
@@ -2565,13 +2461,12 @@
       <c r="G90" s="114" t="n"/>
       <c r="H90" s="114" t="n"/>
       <c r="I90" s="53" t="n"/>
-      <c r="J90" s="55" t="n"/>
+      <c r="J90" s="74" t="n"/>
       <c r="K90" s="74" t="n"/>
-      <c r="L90" s="74" t="n"/>
-      <c r="M90" s="100" t="n"/>
-      <c r="O90" s="92" t="n"/>
+      <c r="L90" s="100" t="n"/>
+      <c r="N90" s="92" t="n"/>
+      <c r="O90" s="57" t="n"/>
       <c r="P90" s="57" t="n"/>
-      <c r="Q90" s="57" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="74" t="n"/>
@@ -2579,13 +2474,12 @@
       <c r="G91" s="114" t="n"/>
       <c r="H91" s="114" t="n"/>
       <c r="I91" s="53" t="n"/>
-      <c r="J91" s="55" t="n"/>
+      <c r="J91" s="74" t="n"/>
       <c r="K91" s="74" t="n"/>
-      <c r="L91" s="74" t="n"/>
-      <c r="M91" s="100" t="n"/>
-      <c r="O91" s="92" t="n"/>
+      <c r="L91" s="100" t="n"/>
+      <c r="N91" s="92" t="n"/>
+      <c r="O91" s="57" t="n"/>
       <c r="P91" s="57" t="n"/>
-      <c r="Q91" s="57" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="74" t="n"/>
@@ -2593,13 +2487,12 @@
       <c r="G92" s="114" t="n"/>
       <c r="H92" s="114" t="n"/>
       <c r="I92" s="53" t="n"/>
-      <c r="J92" s="55" t="n"/>
+      <c r="J92" s="74" t="n"/>
       <c r="K92" s="74" t="n"/>
-      <c r="L92" s="74" t="n"/>
-      <c r="M92" s="100" t="n"/>
-      <c r="O92" s="92" t="n"/>
+      <c r="L92" s="100" t="n"/>
+      <c r="N92" s="92" t="n"/>
+      <c r="O92" s="57" t="n"/>
       <c r="P92" s="57" t="n"/>
-      <c r="Q92" s="57" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="74" t="n"/>
@@ -2607,13 +2500,12 @@
       <c r="G93" s="114" t="n"/>
       <c r="H93" s="114" t="n"/>
       <c r="I93" s="53" t="n"/>
-      <c r="J93" s="55" t="n"/>
+      <c r="J93" s="74" t="n"/>
       <c r="K93" s="74" t="n"/>
-      <c r="L93" s="74" t="n"/>
-      <c r="M93" s="100" t="n"/>
-      <c r="O93" s="92" t="n"/>
+      <c r="L93" s="100" t="n"/>
+      <c r="N93" s="92" t="n"/>
+      <c r="O93" s="57" t="n"/>
       <c r="P93" s="57" t="n"/>
-      <c r="Q93" s="57" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="74" t="n"/>
@@ -2621,13 +2513,12 @@
       <c r="G94" s="114" t="n"/>
       <c r="H94" s="114" t="n"/>
       <c r="I94" s="53" t="n"/>
-      <c r="J94" s="55" t="n"/>
+      <c r="J94" s="74" t="n"/>
       <c r="K94" s="74" t="n"/>
-      <c r="L94" s="74" t="n"/>
-      <c r="M94" s="100" t="n"/>
-      <c r="O94" s="92" t="n"/>
+      <c r="L94" s="100" t="n"/>
+      <c r="N94" s="92" t="n"/>
+      <c r="O94" s="57" t="n"/>
       <c r="P94" s="57" t="n"/>
-      <c r="Q94" s="57" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="74" t="n"/>
@@ -2635,13 +2526,12 @@
       <c r="G95" s="114" t="n"/>
       <c r="H95" s="114" t="n"/>
       <c r="I95" s="53" t="n"/>
-      <c r="J95" s="55" t="n"/>
+      <c r="J95" s="74" t="n"/>
       <c r="K95" s="74" t="n"/>
-      <c r="L95" s="74" t="n"/>
-      <c r="M95" s="100" t="n"/>
-      <c r="O95" s="92" t="n"/>
+      <c r="L95" s="100" t="n"/>
+      <c r="N95" s="92" t="n"/>
+      <c r="O95" s="57" t="n"/>
       <c r="P95" s="57" t="n"/>
-      <c r="Q95" s="57" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="74" t="n"/>
@@ -2652,13 +2542,12 @@
       <c r="G96" s="114" t="n"/>
       <c r="H96" s="50" t="n"/>
       <c r="I96" s="53" t="n"/>
-      <c r="J96" s="55" t="n"/>
+      <c r="J96" s="74" t="n"/>
       <c r="K96" s="74" t="n"/>
-      <c r="L96" s="74" t="n"/>
-      <c r="M96" s="100" t="n"/>
-      <c r="O96" s="92" t="n"/>
+      <c r="L96" s="100" t="n"/>
+      <c r="N96" s="92" t="n"/>
+      <c r="O96" s="57" t="n"/>
       <c r="P96" s="57" t="n"/>
-      <c r="Q96" s="57" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="74" t="n"/>
@@ -2666,13 +2555,12 @@
       <c r="G97" s="114" t="n"/>
       <c r="H97" s="114" t="n"/>
       <c r="I97" s="53" t="n"/>
-      <c r="J97" s="55" t="n"/>
+      <c r="J97" s="74" t="n"/>
       <c r="K97" s="74" t="n"/>
-      <c r="L97" s="74" t="n"/>
-      <c r="M97" s="100" t="n"/>
-      <c r="O97" s="92" t="n"/>
+      <c r="L97" s="100" t="n"/>
+      <c r="N97" s="92" t="n"/>
+      <c r="O97" s="57" t="n"/>
       <c r="P97" s="57" t="n"/>
-      <c r="Q97" s="57" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="74" t="n"/>
@@ -2683,13 +2571,12 @@
       <c r="G98" s="114" t="n"/>
       <c r="H98" s="114" t="n"/>
       <c r="I98" s="53" t="n"/>
-      <c r="J98" s="55" t="n"/>
+      <c r="J98" s="74" t="n"/>
       <c r="K98" s="74" t="n"/>
-      <c r="L98" s="74" t="n"/>
-      <c r="M98" s="100" t="n"/>
-      <c r="O98" s="92" t="n"/>
+      <c r="L98" s="100" t="n"/>
+      <c r="N98" s="92" t="n"/>
+      <c r="O98" s="57" t="n"/>
       <c r="P98" s="57" t="n"/>
-      <c r="Q98" s="57" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="74" t="n"/>
@@ -2697,13 +2584,12 @@
       <c r="G99" s="114" t="n"/>
       <c r="H99" s="114" t="n"/>
       <c r="I99" s="53" t="n"/>
-      <c r="J99" s="55" t="n"/>
+      <c r="J99" s="74" t="n"/>
       <c r="K99" s="74" t="n"/>
-      <c r="L99" s="74" t="n"/>
-      <c r="M99" s="100" t="n"/>
-      <c r="O99" s="92" t="n"/>
+      <c r="L99" s="100" t="n"/>
+      <c r="N99" s="92" t="n"/>
+      <c r="O99" s="57" t="n"/>
       <c r="P99" s="57" t="n"/>
-      <c r="Q99" s="57" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="74" t="n"/>
@@ -2711,13 +2597,12 @@
       <c r="G100" s="114" t="n"/>
       <c r="H100" s="114" t="n"/>
       <c r="I100" s="53" t="n"/>
-      <c r="J100" s="55" t="n"/>
+      <c r="J100" s="74" t="n"/>
       <c r="K100" s="74" t="n"/>
-      <c r="L100" s="74" t="n"/>
-      <c r="M100" s="100" t="n"/>
-      <c r="O100" s="92" t="n"/>
+      <c r="L100" s="100" t="n"/>
+      <c r="N100" s="92" t="n"/>
+      <c r="O100" s="57" t="n"/>
       <c r="P100" s="57" t="n"/>
-      <c r="Q100" s="57" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="74" t="n"/>
@@ -2725,13 +2610,12 @@
       <c r="G101" s="114" t="n"/>
       <c r="H101" s="114" t="n"/>
       <c r="I101" s="53" t="n"/>
-      <c r="J101" s="55" t="n"/>
+      <c r="J101" s="74" t="n"/>
       <c r="K101" s="74" t="n"/>
-      <c r="L101" s="74" t="n"/>
-      <c r="M101" s="100" t="n"/>
-      <c r="O101" s="92" t="n"/>
+      <c r="L101" s="100" t="n"/>
+      <c r="N101" s="92" t="n"/>
+      <c r="O101" s="57" t="n"/>
       <c r="P101" s="57" t="n"/>
-      <c r="Q101" s="57" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="74" t="n"/>
@@ -2739,13 +2623,12 @@
       <c r="G102" s="114" t="n"/>
       <c r="H102" s="114" t="n"/>
       <c r="I102" s="53" t="n"/>
-      <c r="J102" s="55" t="n"/>
+      <c r="J102" s="74" t="n"/>
       <c r="K102" s="74" t="n"/>
-      <c r="L102" s="74" t="n"/>
-      <c r="M102" s="100" t="n"/>
-      <c r="O102" s="92" t="n"/>
+      <c r="L102" s="100" t="n"/>
+      <c r="N102" s="92" t="n"/>
+      <c r="O102" s="57" t="n"/>
       <c r="P102" s="57" t="n"/>
-      <c r="Q102" s="57" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="74" t="n"/>
@@ -2753,13 +2636,12 @@
       <c r="G103" s="114" t="n"/>
       <c r="H103" s="114" t="n"/>
       <c r="I103" s="53" t="n"/>
-      <c r="J103" s="55" t="n"/>
+      <c r="J103" s="74" t="n"/>
       <c r="K103" s="74" t="n"/>
-      <c r="L103" s="74" t="n"/>
-      <c r="M103" s="100" t="n"/>
-      <c r="O103" s="92" t="n"/>
+      <c r="L103" s="100" t="n"/>
+      <c r="N103" s="92" t="n"/>
+      <c r="O103" s="57" t="n"/>
       <c r="P103" s="57" t="n"/>
-      <c r="Q103" s="57" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="74" t="n"/>
@@ -2767,13 +2649,12 @@
       <c r="G104" s="114" t="n"/>
       <c r="H104" s="114" t="n"/>
       <c r="I104" s="53" t="n"/>
-      <c r="J104" s="55" t="n"/>
+      <c r="J104" s="74" t="n"/>
       <c r="K104" s="74" t="n"/>
-      <c r="L104" s="74" t="n"/>
-      <c r="M104" s="100" t="n"/>
-      <c r="O104" s="92" t="n"/>
+      <c r="L104" s="100" t="n"/>
+      <c r="N104" s="92" t="n"/>
+      <c r="O104" s="57" t="n"/>
       <c r="P104" s="57" t="n"/>
-      <c r="Q104" s="57" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="74" t="n"/>
@@ -2781,13 +2662,12 @@
       <c r="G105" s="114" t="n"/>
       <c r="H105" s="114" t="n"/>
       <c r="I105" s="53" t="n"/>
-      <c r="J105" s="55" t="n"/>
+      <c r="J105" s="74" t="n"/>
       <c r="K105" s="74" t="n"/>
-      <c r="L105" s="74" t="n"/>
-      <c r="M105" s="100" t="n"/>
-      <c r="O105" s="92" t="n"/>
+      <c r="L105" s="100" t="n"/>
+      <c r="N105" s="92" t="n"/>
+      <c r="O105" s="57" t="n"/>
       <c r="P105" s="57" t="n"/>
-      <c r="Q105" s="57" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="74" t="n"/>
@@ -2795,13 +2675,12 @@
       <c r="G106" s="114" t="n"/>
       <c r="H106" s="114" t="n"/>
       <c r="I106" s="53" t="n"/>
-      <c r="J106" s="55" t="n"/>
+      <c r="J106" s="74" t="n"/>
       <c r="K106" s="74" t="n"/>
-      <c r="L106" s="74" t="n"/>
-      <c r="M106" s="100" t="n"/>
-      <c r="O106" s="92" t="n"/>
+      <c r="L106" s="100" t="n"/>
+      <c r="N106" s="92" t="n"/>
+      <c r="O106" s="57" t="n"/>
       <c r="P106" s="57" t="n"/>
-      <c r="Q106" s="57" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="74" t="n"/>
@@ -2809,13 +2688,12 @@
       <c r="G107" s="114" t="n"/>
       <c r="H107" s="114" t="n"/>
       <c r="I107" s="53" t="n"/>
-      <c r="J107" s="55" t="n"/>
+      <c r="J107" s="74" t="n"/>
       <c r="K107" s="74" t="n"/>
-      <c r="L107" s="74" t="n"/>
-      <c r="M107" s="100" t="n"/>
-      <c r="O107" s="92" t="n"/>
+      <c r="L107" s="100" t="n"/>
+      <c r="N107" s="92" t="n"/>
+      <c r="O107" s="57" t="n"/>
       <c r="P107" s="57" t="n"/>
-      <c r="Q107" s="57" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="74" t="n"/>
@@ -2823,13 +2701,12 @@
       <c r="G108" s="114" t="n"/>
       <c r="H108" s="114" t="n"/>
       <c r="I108" s="53" t="n"/>
-      <c r="J108" s="55" t="n"/>
+      <c r="J108" s="74" t="n"/>
       <c r="K108" s="74" t="n"/>
-      <c r="L108" s="74" t="n"/>
-      <c r="M108" s="100" t="n"/>
-      <c r="O108" s="92" t="n"/>
+      <c r="L108" s="100" t="n"/>
+      <c r="N108" s="92" t="n"/>
+      <c r="O108" s="57" t="n"/>
       <c r="P108" s="57" t="n"/>
-      <c r="Q108" s="57" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="74" t="n"/>
@@ -2839,13 +2716,12 @@
       <c r="G109" s="114" t="n"/>
       <c r="H109" s="114" t="n"/>
       <c r="I109" s="53" t="n"/>
-      <c r="J109" s="55" t="n"/>
+      <c r="J109" s="74" t="n"/>
       <c r="K109" s="74" t="n"/>
-      <c r="L109" s="74" t="n"/>
-      <c r="M109" s="100" t="n"/>
-      <c r="O109" s="92" t="n"/>
+      <c r="L109" s="100" t="n"/>
+      <c r="N109" s="92" t="n"/>
+      <c r="O109" s="57" t="n"/>
       <c r="P109" s="57" t="n"/>
-      <c r="Q109" s="57" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="74" t="n"/>
@@ -2854,13 +2730,12 @@
       <c r="G110" s="114" t="n"/>
       <c r="H110" s="114" t="n"/>
       <c r="I110" s="53" t="n"/>
-      <c r="J110" s="55" t="n"/>
+      <c r="J110" s="74" t="n"/>
       <c r="K110" s="74" t="n"/>
-      <c r="L110" s="74" t="n"/>
-      <c r="M110" s="100" t="n"/>
-      <c r="O110" s="92" t="n"/>
+      <c r="L110" s="100" t="n"/>
+      <c r="N110" s="92" t="n"/>
+      <c r="O110" s="57" t="n"/>
       <c r="P110" s="57" t="n"/>
-      <c r="Q110" s="57" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="74" t="n"/>
@@ -2869,13 +2744,12 @@
       <c r="G111" s="114" t="n"/>
       <c r="H111" s="114" t="n"/>
       <c r="I111" s="53" t="n"/>
-      <c r="J111" s="55" t="n"/>
+      <c r="J111" s="74" t="n"/>
       <c r="K111" s="74" t="n"/>
-      <c r="L111" s="74" t="n"/>
-      <c r="M111" s="100" t="n"/>
-      <c r="O111" s="92" t="n"/>
+      <c r="L111" s="100" t="n"/>
+      <c r="N111" s="92" t="n"/>
+      <c r="O111" s="57" t="n"/>
       <c r="P111" s="57" t="n"/>
-      <c r="Q111" s="57" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="74" t="n"/>
@@ -2883,13 +2757,12 @@
       <c r="G112" s="114" t="n"/>
       <c r="H112" s="114" t="n"/>
       <c r="I112" s="53" t="n"/>
-      <c r="J112" s="55" t="n"/>
+      <c r="J112" s="74" t="n"/>
       <c r="K112" s="74" t="n"/>
-      <c r="L112" s="74" t="n"/>
-      <c r="M112" s="100" t="n"/>
-      <c r="O112" s="92" t="n"/>
+      <c r="L112" s="100" t="n"/>
+      <c r="N112" s="92" t="n"/>
+      <c r="O112" s="57" t="n"/>
       <c r="P112" s="57" t="n"/>
-      <c r="Q112" s="57" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="74" t="n"/>
@@ -2897,13 +2770,12 @@
       <c r="G113" s="114" t="n"/>
       <c r="H113" s="114" t="n"/>
       <c r="I113" s="53" t="n"/>
-      <c r="J113" s="55" t="n"/>
+      <c r="J113" s="74" t="n"/>
       <c r="K113" s="74" t="n"/>
-      <c r="L113" s="74" t="n"/>
-      <c r="M113" s="100" t="n"/>
-      <c r="O113" s="92" t="n"/>
+      <c r="L113" s="100" t="n"/>
+      <c r="N113" s="92" t="n"/>
+      <c r="O113" s="57" t="n"/>
       <c r="P113" s="57" t="n"/>
-      <c r="Q113" s="57" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="74" t="n"/>
@@ -2912,13 +2784,12 @@
       <c r="G114" s="114" t="n"/>
       <c r="H114" s="114" t="n"/>
       <c r="I114" s="53" t="n"/>
-      <c r="J114" s="55" t="n"/>
+      <c r="J114" s="74" t="n"/>
       <c r="K114" s="74" t="n"/>
-      <c r="L114" s="74" t="n"/>
-      <c r="M114" s="100" t="n"/>
-      <c r="O114" s="92" t="n"/>
+      <c r="L114" s="100" t="n"/>
+      <c r="N114" s="92" t="n"/>
+      <c r="O114" s="57" t="n"/>
       <c r="P114" s="57" t="n"/>
-      <c r="Q114" s="57" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="74" t="n"/>
@@ -2926,13 +2797,12 @@
       <c r="G115" s="114" t="n"/>
       <c r="H115" s="114" t="n"/>
       <c r="I115" s="53" t="n"/>
-      <c r="J115" s="55" t="n"/>
+      <c r="J115" s="74" t="n"/>
       <c r="K115" s="74" t="n"/>
-      <c r="L115" s="74" t="n"/>
-      <c r="M115" s="100" t="n"/>
-      <c r="O115" s="92" t="n"/>
+      <c r="L115" s="100" t="n"/>
+      <c r="N115" s="92" t="n"/>
+      <c r="O115" s="57" t="n"/>
       <c r="P115" s="57" t="n"/>
-      <c r="Q115" s="57" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="74" t="n"/>
@@ -2940,13 +2810,12 @@
       <c r="G116" s="114" t="n"/>
       <c r="H116" s="114" t="n"/>
       <c r="I116" s="53" t="n"/>
-      <c r="J116" s="55" t="n"/>
+      <c r="J116" s="74" t="n"/>
       <c r="K116" s="74" t="n"/>
-      <c r="L116" s="74" t="n"/>
-      <c r="M116" s="100" t="n"/>
-      <c r="O116" s="92" t="n"/>
+      <c r="L116" s="100" t="n"/>
+      <c r="N116" s="92" t="n"/>
+      <c r="O116" s="57" t="n"/>
       <c r="P116" s="57" t="n"/>
-      <c r="Q116" s="57" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="74" t="n"/>
@@ -2955,13 +2824,12 @@
       <c r="G117" s="114" t="n"/>
       <c r="H117" s="114" t="n"/>
       <c r="I117" s="53" t="n"/>
-      <c r="J117" s="55" t="n"/>
+      <c r="J117" s="74" t="n"/>
       <c r="K117" s="74" t="n"/>
-      <c r="L117" s="74" t="n"/>
-      <c r="M117" s="100" t="n"/>
-      <c r="O117" s="92" t="n"/>
+      <c r="L117" s="100" t="n"/>
+      <c r="N117" s="92" t="n"/>
+      <c r="O117" s="57" t="n"/>
       <c r="P117" s="57" t="n"/>
-      <c r="Q117" s="57" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="74" t="n"/>
@@ -2969,13 +2837,12 @@
       <c r="G118" s="114" t="n"/>
       <c r="H118" s="114" t="n"/>
       <c r="I118" s="53" t="n"/>
-      <c r="J118" s="55" t="n"/>
+      <c r="J118" s="74" t="n"/>
       <c r="K118" s="74" t="n"/>
-      <c r="L118" s="74" t="n"/>
-      <c r="M118" s="100" t="n"/>
-      <c r="O118" s="92" t="n"/>
+      <c r="L118" s="100" t="n"/>
+      <c r="N118" s="92" t="n"/>
+      <c r="O118" s="57" t="n"/>
       <c r="P118" s="57" t="n"/>
-      <c r="Q118" s="57" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="74" t="n"/>
@@ -2983,13 +2850,12 @@
       <c r="G119" s="114" t="n"/>
       <c r="H119" s="114" t="n"/>
       <c r="I119" s="53" t="n"/>
-      <c r="J119" s="55" t="n"/>
+      <c r="J119" s="74" t="n"/>
       <c r="K119" s="74" t="n"/>
-      <c r="L119" s="74" t="n"/>
-      <c r="M119" s="100" t="n"/>
-      <c r="O119" s="92" t="n"/>
+      <c r="L119" s="100" t="n"/>
+      <c r="N119" s="92" t="n"/>
+      <c r="O119" s="57" t="n"/>
       <c r="P119" s="57" t="n"/>
-      <c r="Q119" s="57" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="74" t="n"/>
@@ -2998,13 +2864,12 @@
       <c r="G120" s="114" t="n"/>
       <c r="H120" s="114" t="n"/>
       <c r="I120" s="53" t="n"/>
-      <c r="J120" s="55" t="n"/>
+      <c r="J120" s="74" t="n"/>
       <c r="K120" s="74" t="n"/>
-      <c r="L120" s="74" t="n"/>
-      <c r="M120" s="100" t="n"/>
-      <c r="O120" s="92" t="n"/>
+      <c r="L120" s="100" t="n"/>
+      <c r="N120" s="92" t="n"/>
+      <c r="O120" s="57" t="n"/>
       <c r="P120" s="57" t="n"/>
-      <c r="Q120" s="57" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="74" t="n"/>
@@ -3012,13 +2877,12 @@
       <c r="G121" s="114" t="n"/>
       <c r="H121" s="114" t="n"/>
       <c r="I121" s="53" t="n"/>
-      <c r="J121" s="55" t="n"/>
+      <c r="J121" s="74" t="n"/>
       <c r="K121" s="74" t="n"/>
-      <c r="L121" s="74" t="n"/>
-      <c r="M121" s="100" t="n"/>
-      <c r="O121" s="92" t="n"/>
+      <c r="L121" s="100" t="n"/>
+      <c r="N121" s="92" t="n"/>
+      <c r="O121" s="57" t="n"/>
       <c r="P121" s="57" t="n"/>
-      <c r="Q121" s="57" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="74" t="n"/>
@@ -3027,13 +2891,12 @@
       <c r="G122" s="114" t="n"/>
       <c r="H122" s="114" t="n"/>
       <c r="I122" s="53" t="n"/>
-      <c r="J122" s="55" t="n"/>
+      <c r="J122" s="74" t="n"/>
       <c r="K122" s="74" t="n"/>
-      <c r="L122" s="74" t="n"/>
-      <c r="M122" s="100" t="n"/>
-      <c r="O122" s="92" t="n"/>
+      <c r="L122" s="100" t="n"/>
+      <c r="N122" s="92" t="n"/>
+      <c r="O122" s="57" t="n"/>
       <c r="P122" s="57" t="n"/>
-      <c r="Q122" s="57" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="74" t="n"/>
@@ -3041,13 +2904,12 @@
       <c r="G123" s="114" t="n"/>
       <c r="H123" s="114" t="n"/>
       <c r="I123" s="53" t="n"/>
-      <c r="J123" s="55" t="n"/>
+      <c r="J123" s="74" t="n"/>
       <c r="K123" s="74" t="n"/>
-      <c r="L123" s="74" t="n"/>
-      <c r="M123" s="100" t="n"/>
-      <c r="O123" s="92" t="n"/>
+      <c r="L123" s="100" t="n"/>
+      <c r="N123" s="92" t="n"/>
+      <c r="O123" s="57" t="n"/>
       <c r="P123" s="57" t="n"/>
-      <c r="Q123" s="57" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="74" t="n"/>
@@ -3055,39 +2917,36 @@
       <c r="G124" s="114" t="n"/>
       <c r="H124" s="114" t="n"/>
       <c r="I124" s="53" t="n"/>
-      <c r="J124" s="55" t="n"/>
+      <c r="J124" s="74" t="n"/>
       <c r="K124" s="74" t="n"/>
-      <c r="L124" s="74" t="n"/>
-      <c r="M124" s="100" t="n"/>
-      <c r="O124" s="92" t="n"/>
+      <c r="L124" s="100" t="n"/>
+      <c r="N124" s="92" t="n"/>
+      <c r="O124" s="57" t="n"/>
       <c r="P124" s="57" t="n"/>
-      <c r="Q124" s="57" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="74" t="n"/>
       <c r="G125" s="114" t="n"/>
       <c r="H125" s="114" t="n"/>
       <c r="I125" s="53" t="n"/>
-      <c r="J125" s="55" t="n"/>
+      <c r="J125" s="74" t="n"/>
       <c r="K125" s="74" t="n"/>
-      <c r="L125" s="74" t="n"/>
-      <c r="M125" s="100" t="n"/>
-      <c r="O125" s="92" t="n"/>
+      <c r="L125" s="100" t="n"/>
+      <c r="N125" s="92" t="n"/>
+      <c r="O125" s="57" t="n"/>
       <c r="P125" s="57" t="n"/>
-      <c r="Q125" s="57" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="74" t="n"/>
       <c r="G126" s="114" t="n"/>
       <c r="H126" s="114" t="n"/>
       <c r="I126" s="53" t="n"/>
-      <c r="J126" s="55" t="n"/>
+      <c r="J126" s="74" t="n"/>
       <c r="K126" s="74" t="n"/>
-      <c r="L126" s="74" t="n"/>
-      <c r="M126" s="100" t="n"/>
-      <c r="O126" s="92" t="n"/>
+      <c r="L126" s="100" t="n"/>
+      <c r="N126" s="92" t="n"/>
+      <c r="O126" s="57" t="n"/>
       <c r="P126" s="57" t="n"/>
-      <c r="Q126" s="57" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="74" t="n"/>
@@ -3095,13 +2954,12 @@
       <c r="G127" s="114" t="n"/>
       <c r="H127" s="114" t="n"/>
       <c r="I127" s="53" t="n"/>
-      <c r="J127" s="55" t="n"/>
+      <c r="J127" s="74" t="n"/>
       <c r="K127" s="74" t="n"/>
-      <c r="L127" s="74" t="n"/>
-      <c r="M127" s="100" t="n"/>
-      <c r="O127" s="92" t="n"/>
+      <c r="L127" s="100" t="n"/>
+      <c r="N127" s="92" t="n"/>
+      <c r="O127" s="57" t="n"/>
       <c r="P127" s="57" t="n"/>
-      <c r="Q127" s="57" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="74" t="n"/>
@@ -3110,13 +2968,12 @@
       <c r="G128" s="114" t="n"/>
       <c r="H128" s="114" t="n"/>
       <c r="I128" s="53" t="n"/>
-      <c r="J128" s="55" t="n"/>
+      <c r="J128" s="74" t="n"/>
       <c r="K128" s="74" t="n"/>
-      <c r="L128" s="74" t="n"/>
-      <c r="M128" s="100" t="n"/>
-      <c r="O128" s="92" t="n"/>
+      <c r="L128" s="100" t="n"/>
+      <c r="N128" s="92" t="n"/>
+      <c r="O128" s="57" t="n"/>
       <c r="P128" s="57" t="n"/>
-      <c r="Q128" s="57" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="74" t="n"/>
@@ -3124,13 +2981,12 @@
       <c r="G129" s="114" t="n"/>
       <c r="H129" s="114" t="n"/>
       <c r="I129" s="53" t="n"/>
-      <c r="J129" s="55" t="n"/>
+      <c r="J129" s="74" t="n"/>
       <c r="K129" s="74" t="n"/>
-      <c r="L129" s="74" t="n"/>
-      <c r="M129" s="100" t="n"/>
-      <c r="O129" s="92" t="n"/>
+      <c r="L129" s="100" t="n"/>
+      <c r="N129" s="92" t="n"/>
+      <c r="O129" s="57" t="n"/>
       <c r="P129" s="57" t="n"/>
-      <c r="Q129" s="57" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="74" t="n"/>
@@ -3138,13 +2994,12 @@
       <c r="G130" s="114" t="n"/>
       <c r="H130" s="114" t="n"/>
       <c r="I130" s="53" t="n"/>
-      <c r="J130" s="55" t="n"/>
+      <c r="J130" s="74" t="n"/>
       <c r="K130" s="74" t="n"/>
-      <c r="L130" s="74" t="n"/>
-      <c r="M130" s="100" t="n"/>
-      <c r="O130" s="92" t="n"/>
+      <c r="L130" s="100" t="n"/>
+      <c r="N130" s="92" t="n"/>
+      <c r="O130" s="57" t="n"/>
       <c r="P130" s="57" t="n"/>
-      <c r="Q130" s="57" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="74" t="n"/>
@@ -3152,13 +3007,12 @@
       <c r="G131" s="114" t="n"/>
       <c r="H131" s="114" t="n"/>
       <c r="I131" s="53" t="n"/>
-      <c r="J131" s="55" t="n"/>
+      <c r="J131" s="74" t="n"/>
       <c r="K131" s="74" t="n"/>
-      <c r="L131" s="74" t="n"/>
-      <c r="M131" s="100" t="n"/>
-      <c r="O131" s="92" t="n"/>
+      <c r="L131" s="100" t="n"/>
+      <c r="N131" s="92" t="n"/>
+      <c r="O131" s="57" t="n"/>
       <c r="P131" s="57" t="n"/>
-      <c r="Q131" s="57" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="74" t="n"/>
@@ -3166,13 +3020,12 @@
       <c r="G132" s="114" t="n"/>
       <c r="H132" s="114" t="n"/>
       <c r="I132" s="53" t="n"/>
-      <c r="J132" s="55" t="n"/>
+      <c r="J132" s="74" t="n"/>
       <c r="K132" s="74" t="n"/>
-      <c r="L132" s="74" t="n"/>
-      <c r="M132" s="100" t="n"/>
-      <c r="O132" s="92" t="n"/>
+      <c r="L132" s="100" t="n"/>
+      <c r="N132" s="92" t="n"/>
+      <c r="O132" s="57" t="n"/>
       <c r="P132" s="57" t="n"/>
-      <c r="Q132" s="57" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="74" t="n"/>
@@ -3180,13 +3033,12 @@
       <c r="G133" s="114" t="n"/>
       <c r="H133" s="114" t="n"/>
       <c r="I133" s="53" t="n"/>
-      <c r="J133" s="55" t="n"/>
+      <c r="J133" s="74" t="n"/>
       <c r="K133" s="74" t="n"/>
-      <c r="L133" s="74" t="n"/>
-      <c r="M133" s="100" t="n"/>
-      <c r="O133" s="92" t="n"/>
+      <c r="L133" s="100" t="n"/>
+      <c r="N133" s="92" t="n"/>
+      <c r="O133" s="57" t="n"/>
       <c r="P133" s="57" t="n"/>
-      <c r="Q133" s="57" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="74" t="n"/>
@@ -3194,26 +3046,24 @@
       <c r="G134" s="114" t="n"/>
       <c r="H134" s="114" t="n"/>
       <c r="I134" s="53" t="n"/>
-      <c r="J134" s="55" t="n"/>
+      <c r="J134" s="74" t="n"/>
       <c r="K134" s="74" t="n"/>
-      <c r="L134" s="74" t="n"/>
-      <c r="M134" s="100" t="n"/>
-      <c r="O134" s="92" t="n"/>
+      <c r="L134" s="100" t="n"/>
+      <c r="N134" s="92" t="n"/>
+      <c r="O134" s="57" t="n"/>
       <c r="P134" s="57" t="n"/>
-      <c r="Q134" s="57" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="74" t="n"/>
       <c r="G135" s="114" t="n"/>
       <c r="H135" s="114" t="n"/>
       <c r="I135" s="53" t="n"/>
-      <c r="J135" s="55" t="n"/>
+      <c r="J135" s="74" t="n"/>
       <c r="K135" s="74" t="n"/>
-      <c r="L135" s="74" t="n"/>
-      <c r="M135" s="100" t="n"/>
-      <c r="O135" s="92" t="n"/>
+      <c r="L135" s="100" t="n"/>
+      <c r="N135" s="92" t="n"/>
+      <c r="O135" s="57" t="n"/>
       <c r="P135" s="57" t="n"/>
-      <c r="Q135" s="57" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="74" t="n"/>
@@ -3221,26 +3071,24 @@
       <c r="G136" s="114" t="n"/>
       <c r="H136" s="114" t="n"/>
       <c r="I136" s="53" t="n"/>
-      <c r="J136" s="55" t="n"/>
+      <c r="J136" s="74" t="n"/>
       <c r="K136" s="74" t="n"/>
-      <c r="L136" s="74" t="n"/>
-      <c r="M136" s="100" t="n"/>
-      <c r="O136" s="92" t="n"/>
+      <c r="L136" s="100" t="n"/>
+      <c r="N136" s="92" t="n"/>
+      <c r="O136" s="57" t="n"/>
       <c r="P136" s="57" t="n"/>
-      <c r="Q136" s="57" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="74" t="n"/>
       <c r="G137" s="114" t="n"/>
       <c r="H137" s="114" t="n"/>
       <c r="I137" s="53" t="n"/>
-      <c r="J137" s="55" t="n"/>
+      <c r="J137" s="74" t="n"/>
       <c r="K137" s="74" t="n"/>
-      <c r="L137" s="74" t="n"/>
-      <c r="M137" s="100" t="n"/>
-      <c r="O137" s="92" t="n"/>
+      <c r="L137" s="100" t="n"/>
+      <c r="N137" s="92" t="n"/>
+      <c r="O137" s="57" t="n"/>
       <c r="P137" s="57" t="n"/>
-      <c r="Q137" s="57" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="74" t="n"/>
@@ -3248,13 +3096,12 @@
       <c r="G138" s="114" t="n"/>
       <c r="H138" s="114" t="n"/>
       <c r="I138" s="53" t="n"/>
-      <c r="J138" s="55" t="n"/>
+      <c r="J138" s="74" t="n"/>
       <c r="K138" s="74" t="n"/>
-      <c r="L138" s="74" t="n"/>
-      <c r="M138" s="100" t="n"/>
-      <c r="O138" s="92" t="n"/>
+      <c r="L138" s="100" t="n"/>
+      <c r="N138" s="92" t="n"/>
+      <c r="O138" s="57" t="n"/>
       <c r="P138" s="57" t="n"/>
-      <c r="Q138" s="57" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="74" t="n"/>
@@ -3262,13 +3109,12 @@
       <c r="G139" s="114" t="n"/>
       <c r="H139" s="114" t="n"/>
       <c r="I139" s="53" t="n"/>
-      <c r="J139" s="55" t="n"/>
+      <c r="J139" s="74" t="n"/>
       <c r="K139" s="74" t="n"/>
-      <c r="L139" s="74" t="n"/>
-      <c r="M139" s="100" t="n"/>
-      <c r="O139" s="92" t="n"/>
+      <c r="L139" s="100" t="n"/>
+      <c r="N139" s="92" t="n"/>
+      <c r="O139" s="57" t="n"/>
       <c r="P139" s="57" t="n"/>
-      <c r="Q139" s="57" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="74" t="n"/>
@@ -3276,13 +3122,12 @@
       <c r="G140" s="114" t="n"/>
       <c r="H140" s="114" t="n"/>
       <c r="I140" s="53" t="n"/>
-      <c r="J140" s="55" t="n"/>
+      <c r="J140" s="74" t="n"/>
       <c r="K140" s="74" t="n"/>
-      <c r="L140" s="74" t="n"/>
-      <c r="M140" s="100" t="n"/>
-      <c r="O140" s="92" t="n"/>
+      <c r="L140" s="100" t="n"/>
+      <c r="N140" s="92" t="n"/>
+      <c r="O140" s="57" t="n"/>
       <c r="P140" s="57" t="n"/>
-      <c r="Q140" s="57" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="74" t="n"/>
@@ -3290,13 +3135,12 @@
       <c r="G141" s="114" t="n"/>
       <c r="H141" s="114" t="n"/>
       <c r="I141" s="53" t="n"/>
-      <c r="J141" s="55" t="n"/>
+      <c r="J141" s="74" t="n"/>
       <c r="K141" s="74" t="n"/>
-      <c r="L141" s="74" t="n"/>
-      <c r="M141" s="100" t="n"/>
-      <c r="O141" s="92" t="n"/>
+      <c r="L141" s="100" t="n"/>
+      <c r="N141" s="92" t="n"/>
+      <c r="O141" s="57" t="n"/>
       <c r="P141" s="57" t="n"/>
-      <c r="Q141" s="57" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="74" t="n"/>
@@ -3304,13 +3148,12 @@
       <c r="G142" s="114" t="n"/>
       <c r="H142" s="114" t="n"/>
       <c r="I142" s="53" t="n"/>
-      <c r="J142" s="55" t="n"/>
+      <c r="J142" s="74" t="n"/>
       <c r="K142" s="74" t="n"/>
-      <c r="L142" s="74" t="n"/>
-      <c r="M142" s="100" t="n"/>
-      <c r="O142" s="92" t="n"/>
+      <c r="L142" s="100" t="n"/>
+      <c r="N142" s="92" t="n"/>
+      <c r="O142" s="57" t="n"/>
       <c r="P142" s="57" t="n"/>
-      <c r="Q142" s="57" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="74" t="n"/>
@@ -3318,13 +3161,12 @@
       <c r="G143" s="114" t="n"/>
       <c r="H143" s="114" t="n"/>
       <c r="I143" s="53" t="n"/>
-      <c r="J143" s="55" t="n"/>
+      <c r="J143" s="74" t="n"/>
       <c r="K143" s="74" t="n"/>
-      <c r="L143" s="74" t="n"/>
-      <c r="M143" s="100" t="n"/>
-      <c r="O143" s="92" t="n"/>
+      <c r="L143" s="100" t="n"/>
+      <c r="N143" s="92" t="n"/>
+      <c r="O143" s="57" t="n"/>
       <c r="P143" s="57" t="n"/>
-      <c r="Q143" s="57" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="74" t="n"/>
@@ -3334,13 +3176,12 @@
       <c r="G144" s="114" t="n"/>
       <c r="H144" s="114" t="n"/>
       <c r="I144" s="53" t="n"/>
-      <c r="J144" s="55" t="n"/>
+      <c r="J144" s="74" t="n"/>
       <c r="K144" s="74" t="n"/>
-      <c r="L144" s="74" t="n"/>
-      <c r="M144" s="100" t="n"/>
-      <c r="O144" s="92" t="n"/>
+      <c r="L144" s="100" t="n"/>
+      <c r="N144" s="92" t="n"/>
+      <c r="O144" s="57" t="n"/>
       <c r="P144" s="57" t="n"/>
-      <c r="Q144" s="57" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="74" t="n"/>
@@ -3348,26 +3189,24 @@
       <c r="G145" s="114" t="n"/>
       <c r="H145" s="114" t="n"/>
       <c r="I145" s="53" t="n"/>
-      <c r="J145" s="55" t="n"/>
+      <c r="J145" s="74" t="n"/>
       <c r="K145" s="74" t="n"/>
-      <c r="L145" s="74" t="n"/>
-      <c r="M145" s="100" t="n"/>
-      <c r="O145" s="92" t="n"/>
+      <c r="L145" s="100" t="n"/>
+      <c r="N145" s="92" t="n"/>
+      <c r="O145" s="57" t="n"/>
       <c r="P145" s="57" t="n"/>
-      <c r="Q145" s="57" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="74" t="n"/>
       <c r="G146" s="114" t="n"/>
       <c r="H146" s="114" t="n"/>
       <c r="I146" s="53" t="n"/>
-      <c r="J146" s="55" t="n"/>
+      <c r="J146" s="74" t="n"/>
       <c r="K146" s="74" t="n"/>
-      <c r="L146" s="74" t="n"/>
-      <c r="M146" s="100" t="n"/>
-      <c r="O146" s="92" t="n"/>
+      <c r="L146" s="100" t="n"/>
+      <c r="N146" s="92" t="n"/>
+      <c r="O146" s="57" t="n"/>
       <c r="P146" s="57" t="n"/>
-      <c r="Q146" s="57" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="74" t="n"/>
@@ -3375,13 +3214,12 @@
       <c r="G147" s="114" t="n"/>
       <c r="H147" s="93" t="n"/>
       <c r="I147" s="53" t="n"/>
-      <c r="J147" s="55" t="n"/>
+      <c r="J147" s="74" t="n"/>
       <c r="K147" s="74" t="n"/>
-      <c r="L147" s="74" t="n"/>
-      <c r="M147" s="100" t="n"/>
-      <c r="O147" s="92" t="n"/>
+      <c r="L147" s="100" t="n"/>
+      <c r="N147" s="92" t="n"/>
+      <c r="O147" s="57" t="n"/>
       <c r="P147" s="57" t="n"/>
-      <c r="Q147" s="57" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="74" t="n"/>
@@ -3389,26 +3227,24 @@
       <c r="G148" s="114" t="n"/>
       <c r="H148" s="114" t="n"/>
       <c r="I148" s="53" t="n"/>
-      <c r="J148" s="55" t="n"/>
+      <c r="J148" s="74" t="n"/>
       <c r="K148" s="74" t="n"/>
-      <c r="L148" s="74" t="n"/>
-      <c r="M148" s="100" t="n"/>
-      <c r="O148" s="92" t="n"/>
+      <c r="L148" s="100" t="n"/>
+      <c r="N148" s="92" t="n"/>
+      <c r="O148" s="57" t="n"/>
       <c r="P148" s="57" t="n"/>
-      <c r="Q148" s="57" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="74" t="n"/>
       <c r="G149" s="114" t="n"/>
       <c r="H149" s="114" t="n"/>
       <c r="I149" s="53" t="n"/>
-      <c r="J149" s="55" t="n"/>
+      <c r="J149" s="74" t="n"/>
       <c r="K149" s="74" t="n"/>
-      <c r="L149" s="74" t="n"/>
-      <c r="M149" s="100" t="n"/>
-      <c r="O149" s="92" t="n"/>
+      <c r="L149" s="100" t="n"/>
+      <c r="N149" s="92" t="n"/>
+      <c r="O149" s="57" t="n"/>
       <c r="P149" s="57" t="n"/>
-      <c r="Q149" s="57" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="74" t="n"/>
@@ -3416,13 +3252,12 @@
       <c r="G150" s="114" t="n"/>
       <c r="H150" s="114" t="n"/>
       <c r="I150" s="53" t="n"/>
-      <c r="J150" s="55" t="n"/>
+      <c r="J150" s="74" t="n"/>
       <c r="K150" s="74" t="n"/>
-      <c r="L150" s="74" t="n"/>
-      <c r="M150" s="100" t="n"/>
-      <c r="O150" s="92" t="n"/>
+      <c r="L150" s="100" t="n"/>
+      <c r="N150" s="92" t="n"/>
+      <c r="O150" s="57" t="n"/>
       <c r="P150" s="57" t="n"/>
-      <c r="Q150" s="57" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="74" t="n"/>
@@ -3430,13 +3265,12 @@
       <c r="G151" s="114" t="n"/>
       <c r="H151" s="114" t="n"/>
       <c r="I151" s="53" t="n"/>
-      <c r="J151" s="55" t="n"/>
+      <c r="J151" s="74" t="n"/>
       <c r="K151" s="74" t="n"/>
-      <c r="L151" s="74" t="n"/>
-      <c r="M151" s="100" t="n"/>
-      <c r="O151" s="92" t="n"/>
+      <c r="L151" s="100" t="n"/>
+      <c r="N151" s="92" t="n"/>
+      <c r="O151" s="57" t="n"/>
       <c r="P151" s="57" t="n"/>
-      <c r="Q151" s="57" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="74" t="n"/>
@@ -3444,13 +3278,12 @@
       <c r="G152" s="114" t="n"/>
       <c r="H152" s="114" t="n"/>
       <c r="I152" s="53" t="n"/>
-      <c r="J152" s="55" t="n"/>
+      <c r="J152" s="74" t="n"/>
       <c r="K152" s="74" t="n"/>
-      <c r="L152" s="74" t="n"/>
-      <c r="M152" s="100" t="n"/>
-      <c r="O152" s="92" t="n"/>
+      <c r="L152" s="100" t="n"/>
+      <c r="N152" s="92" t="n"/>
+      <c r="O152" s="57" t="n"/>
       <c r="P152" s="57" t="n"/>
-      <c r="Q152" s="57" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="74" t="n"/>
@@ -3458,26 +3291,24 @@
       <c r="G153" s="114" t="n"/>
       <c r="H153" s="114" t="n"/>
       <c r="I153" s="53" t="n"/>
-      <c r="J153" s="55" t="n"/>
+      <c r="J153" s="74" t="n"/>
       <c r="K153" s="74" t="n"/>
-      <c r="L153" s="74" t="n"/>
-      <c r="M153" s="100" t="n"/>
-      <c r="O153" s="92" t="n"/>
+      <c r="L153" s="100" t="n"/>
+      <c r="N153" s="92" t="n"/>
+      <c r="O153" s="57" t="n"/>
       <c r="P153" s="57" t="n"/>
-      <c r="Q153" s="57" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="74" t="n"/>
       <c r="G154" s="114" t="n"/>
       <c r="H154" s="114" t="n"/>
       <c r="I154" s="53" t="n"/>
-      <c r="J154" s="55" t="n"/>
+      <c r="J154" s="74" t="n"/>
       <c r="K154" s="74" t="n"/>
-      <c r="L154" s="74" t="n"/>
-      <c r="M154" s="100" t="n"/>
-      <c r="O154" s="92" t="n"/>
+      <c r="L154" s="100" t="n"/>
+      <c r="N154" s="92" t="n"/>
+      <c r="O154" s="57" t="n"/>
       <c r="P154" s="57" t="n"/>
-      <c r="Q154" s="57" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="74" t="n"/>
@@ -3485,26 +3316,24 @@
       <c r="G155" s="114" t="n"/>
       <c r="H155" s="114" t="n"/>
       <c r="I155" s="53" t="n"/>
-      <c r="J155" s="55" t="n"/>
+      <c r="J155" s="74" t="n"/>
       <c r="K155" s="74" t="n"/>
-      <c r="L155" s="74" t="n"/>
-      <c r="M155" s="100" t="n"/>
-      <c r="O155" s="92" t="n"/>
+      <c r="L155" s="100" t="n"/>
+      <c r="N155" s="92" t="n"/>
+      <c r="O155" s="57" t="n"/>
       <c r="P155" s="57" t="n"/>
-      <c r="Q155" s="57" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="74" t="n"/>
       <c r="G156" s="114" t="n"/>
       <c r="H156" s="114" t="n"/>
       <c r="I156" s="53" t="n"/>
-      <c r="J156" s="55" t="n"/>
+      <c r="J156" s="74" t="n"/>
       <c r="K156" s="74" t="n"/>
-      <c r="L156" s="74" t="n"/>
-      <c r="M156" s="100" t="n"/>
-      <c r="O156" s="92" t="n"/>
+      <c r="L156" s="100" t="n"/>
+      <c r="N156" s="92" t="n"/>
+      <c r="O156" s="57" t="n"/>
       <c r="P156" s="57" t="n"/>
-      <c r="Q156" s="57" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="74" t="n"/>
@@ -3514,13 +3343,12 @@
       <c r="G157" s="114" t="n"/>
       <c r="H157" s="114" t="n"/>
       <c r="I157" s="53" t="n"/>
-      <c r="J157" s="55" t="n"/>
+      <c r="J157" s="74" t="n"/>
       <c r="K157" s="74" t="n"/>
-      <c r="L157" s="74" t="n"/>
-      <c r="M157" s="100" t="n"/>
-      <c r="O157" s="92" t="n"/>
+      <c r="L157" s="100" t="n"/>
+      <c r="N157" s="92" t="n"/>
+      <c r="O157" s="57" t="n"/>
       <c r="P157" s="57" t="n"/>
-      <c r="Q157" s="57" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="74" t="n"/>
@@ -3529,13 +3357,12 @@
       <c r="G158" s="114" t="n"/>
       <c r="H158" s="114" t="n"/>
       <c r="I158" s="53" t="n"/>
-      <c r="J158" s="55" t="n"/>
+      <c r="J158" s="74" t="n"/>
       <c r="K158" s="74" t="n"/>
-      <c r="L158" s="74" t="n"/>
-      <c r="M158" s="100" t="n"/>
-      <c r="O158" s="92" t="n"/>
+      <c r="L158" s="100" t="n"/>
+      <c r="N158" s="92" t="n"/>
+      <c r="O158" s="57" t="n"/>
       <c r="P158" s="57" t="n"/>
-      <c r="Q158" s="57" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="74" t="n"/>
@@ -3544,13 +3371,12 @@
       <c r="G159" s="114" t="n"/>
       <c r="H159" s="114" t="n"/>
       <c r="I159" s="53" t="n"/>
-      <c r="J159" s="55" t="n"/>
+      <c r="J159" s="74" t="n"/>
       <c r="K159" s="74" t="n"/>
-      <c r="L159" s="74" t="n"/>
-      <c r="M159" s="100" t="n"/>
-      <c r="O159" s="92" t="n"/>
+      <c r="L159" s="100" t="n"/>
+      <c r="N159" s="92" t="n"/>
+      <c r="O159" s="57" t="n"/>
       <c r="P159" s="57" t="n"/>
-      <c r="Q159" s="57" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="74" t="n"/>
@@ -3558,13 +3384,12 @@
       <c r="G160" s="114" t="n"/>
       <c r="H160" s="114" t="n"/>
       <c r="I160" s="53" t="n"/>
-      <c r="J160" s="55" t="n"/>
+      <c r="J160" s="74" t="n"/>
       <c r="K160" s="74" t="n"/>
-      <c r="L160" s="74" t="n"/>
-      <c r="M160" s="100" t="n"/>
-      <c r="O160" s="92" t="n"/>
+      <c r="L160" s="100" t="n"/>
+      <c r="N160" s="92" t="n"/>
+      <c r="O160" s="57" t="n"/>
       <c r="P160" s="57" t="n"/>
-      <c r="Q160" s="57" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="74" t="n"/>
@@ -3572,13 +3397,12 @@
       <c r="G161" s="114" t="n"/>
       <c r="H161" s="114" t="n"/>
       <c r="I161" s="53" t="n"/>
-      <c r="J161" s="55" t="n"/>
+      <c r="J161" s="74" t="n"/>
       <c r="K161" s="74" t="n"/>
-      <c r="L161" s="74" t="n"/>
-      <c r="M161" s="100" t="n"/>
-      <c r="O161" s="92" t="n"/>
+      <c r="L161" s="100" t="n"/>
+      <c r="N161" s="92" t="n"/>
+      <c r="O161" s="57" t="n"/>
       <c r="P161" s="57" t="n"/>
-      <c r="Q161" s="57" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="74" t="n"/>
@@ -3587,26 +3411,24 @@
       <c r="G162" s="114" t="n"/>
       <c r="H162" s="114" t="n"/>
       <c r="I162" s="53" t="n"/>
-      <c r="J162" s="55" t="n"/>
+      <c r="J162" s="74" t="n"/>
       <c r="K162" s="74" t="n"/>
-      <c r="L162" s="74" t="n"/>
-      <c r="M162" s="100" t="n"/>
-      <c r="O162" s="92" t="n"/>
+      <c r="L162" s="100" t="n"/>
+      <c r="N162" s="92" t="n"/>
+      <c r="O162" s="57" t="n"/>
       <c r="P162" s="57" t="n"/>
-      <c r="Q162" s="57" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="74" t="n"/>
       <c r="G163" s="114" t="n"/>
       <c r="H163" s="114" t="n"/>
       <c r="I163" s="53" t="n"/>
-      <c r="J163" s="55" t="n"/>
+      <c r="J163" s="74" t="n"/>
       <c r="K163" s="74" t="n"/>
-      <c r="L163" s="74" t="n"/>
-      <c r="M163" s="100" t="n"/>
-      <c r="O163" s="92" t="n"/>
+      <c r="L163" s="100" t="n"/>
+      <c r="N163" s="92" t="n"/>
+      <c r="O163" s="57" t="n"/>
       <c r="P163" s="57" t="n"/>
-      <c r="Q163" s="57" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="74" t="n"/>
@@ -3614,13 +3436,12 @@
       <c r="G164" s="114" t="n"/>
       <c r="H164" s="114" t="n"/>
       <c r="I164" s="53" t="n"/>
-      <c r="J164" s="55" t="n"/>
+      <c r="J164" s="74" t="n"/>
       <c r="K164" s="74" t="n"/>
-      <c r="L164" s="74" t="n"/>
-      <c r="M164" s="100" t="n"/>
-      <c r="O164" s="92" t="n"/>
+      <c r="L164" s="100" t="n"/>
+      <c r="N164" s="92" t="n"/>
+      <c r="O164" s="57" t="n"/>
       <c r="P164" s="57" t="n"/>
-      <c r="Q164" s="57" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="74" t="n"/>
@@ -3628,13 +3449,12 @@
       <c r="G165" s="114" t="n"/>
       <c r="H165" s="114" t="n"/>
       <c r="I165" s="53" t="n"/>
-      <c r="J165" s="55" t="n"/>
+      <c r="J165" s="74" t="n"/>
       <c r="K165" s="74" t="n"/>
-      <c r="L165" s="74" t="n"/>
-      <c r="M165" s="100" t="n"/>
-      <c r="O165" s="92" t="n"/>
+      <c r="L165" s="100" t="n"/>
+      <c r="N165" s="92" t="n"/>
+      <c r="O165" s="57" t="n"/>
       <c r="P165" s="57" t="n"/>
-      <c r="Q165" s="57" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="74" t="n"/>
@@ -3642,13 +3462,12 @@
       <c r="G166" s="114" t="n"/>
       <c r="H166" s="114" t="n"/>
       <c r="I166" s="53" t="n"/>
-      <c r="J166" s="55" t="n"/>
+      <c r="J166" s="74" t="n"/>
       <c r="K166" s="74" t="n"/>
-      <c r="L166" s="74" t="n"/>
-      <c r="M166" s="100" t="n"/>
-      <c r="O166" s="92" t="n"/>
+      <c r="L166" s="100" t="n"/>
+      <c r="N166" s="92" t="n"/>
+      <c r="O166" s="57" t="n"/>
       <c r="P166" s="57" t="n"/>
-      <c r="Q166" s="57" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="74" t="n"/>
@@ -3658,13 +3477,12 @@
       <c r="G167" s="114" t="n"/>
       <c r="H167" s="114" t="n"/>
       <c r="I167" s="53" t="n"/>
-      <c r="J167" s="55" t="n"/>
+      <c r="J167" s="74" t="n"/>
       <c r="K167" s="74" t="n"/>
-      <c r="L167" s="74" t="n"/>
-      <c r="M167" s="100" t="n"/>
-      <c r="O167" s="92" t="n"/>
+      <c r="L167" s="100" t="n"/>
+      <c r="N167" s="92" t="n"/>
+      <c r="O167" s="57" t="n"/>
       <c r="P167" s="57" t="n"/>
-      <c r="Q167" s="57" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="74" t="n"/>
@@ -3673,13 +3491,12 @@
       <c r="G168" s="114" t="n"/>
       <c r="H168" s="114" t="n"/>
       <c r="I168" s="53" t="n"/>
-      <c r="J168" s="55" t="n"/>
+      <c r="J168" s="74" t="n"/>
       <c r="K168" s="74" t="n"/>
-      <c r="L168" s="74" t="n"/>
-      <c r="M168" s="100" t="n"/>
-      <c r="O168" s="92" t="n"/>
+      <c r="L168" s="100" t="n"/>
+      <c r="N168" s="92" t="n"/>
+      <c r="O168" s="57" t="n"/>
       <c r="P168" s="57" t="n"/>
-      <c r="Q168" s="57" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="74" t="n"/>
@@ -3687,13 +3504,12 @@
       <c r="G169" s="114" t="n"/>
       <c r="H169" s="114" t="n"/>
       <c r="I169" s="53" t="n"/>
-      <c r="J169" s="55" t="n"/>
+      <c r="J169" s="74" t="n"/>
       <c r="K169" s="74" t="n"/>
-      <c r="L169" s="74" t="n"/>
-      <c r="M169" s="100" t="n"/>
-      <c r="O169" s="92" t="n"/>
+      <c r="L169" s="100" t="n"/>
+      <c r="N169" s="92" t="n"/>
+      <c r="O169" s="57" t="n"/>
       <c r="P169" s="57" t="n"/>
-      <c r="Q169" s="57" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="74" t="n"/>
@@ -3701,13 +3517,12 @@
       <c r="G170" s="114" t="n"/>
       <c r="H170" s="114" t="n"/>
       <c r="I170" s="53" t="n"/>
-      <c r="J170" s="55" t="n"/>
+      <c r="J170" s="74" t="n"/>
       <c r="K170" s="74" t="n"/>
-      <c r="L170" s="74" t="n"/>
-      <c r="M170" s="100" t="n"/>
-      <c r="O170" s="92" t="n"/>
+      <c r="L170" s="100" t="n"/>
+      <c r="N170" s="92" t="n"/>
+      <c r="O170" s="57" t="n"/>
       <c r="P170" s="57" t="n"/>
-      <c r="Q170" s="57" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="74" t="n"/>
@@ -3716,13 +3531,12 @@
       <c r="G171" s="114" t="n"/>
       <c r="H171" s="114" t="n"/>
       <c r="I171" s="53" t="n"/>
-      <c r="J171" s="55" t="n"/>
+      <c r="J171" s="74" t="n"/>
       <c r="K171" s="74" t="n"/>
-      <c r="L171" s="74" t="n"/>
-      <c r="M171" s="100" t="n"/>
-      <c r="O171" s="92" t="n"/>
+      <c r="L171" s="100" t="n"/>
+      <c r="N171" s="92" t="n"/>
+      <c r="O171" s="57" t="n"/>
       <c r="P171" s="57" t="n"/>
-      <c r="Q171" s="57" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="74" t="n"/>
@@ -3730,13 +3544,12 @@
       <c r="G172" s="114" t="n"/>
       <c r="H172" s="114" t="n"/>
       <c r="I172" s="53" t="n"/>
-      <c r="J172" s="55" t="n"/>
+      <c r="J172" s="74" t="n"/>
       <c r="K172" s="74" t="n"/>
-      <c r="L172" s="74" t="n"/>
-      <c r="M172" s="100" t="n"/>
-      <c r="O172" s="92" t="n"/>
+      <c r="L172" s="100" t="n"/>
+      <c r="N172" s="92" t="n"/>
+      <c r="O172" s="57" t="n"/>
       <c r="P172" s="57" t="n"/>
-      <c r="Q172" s="57" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="74" t="n"/>
@@ -3744,13 +3557,12 @@
       <c r="G173" s="114" t="n"/>
       <c r="H173" s="114" t="n"/>
       <c r="I173" s="53" t="n"/>
-      <c r="J173" s="55" t="n"/>
+      <c r="J173" s="74" t="n"/>
       <c r="K173" s="74" t="n"/>
-      <c r="L173" s="74" t="n"/>
-      <c r="M173" s="100" t="n"/>
-      <c r="O173" s="92" t="n"/>
+      <c r="L173" s="100" t="n"/>
+      <c r="N173" s="92" t="n"/>
+      <c r="O173" s="57" t="n"/>
       <c r="P173" s="57" t="n"/>
-      <c r="Q173" s="57" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="74" t="n"/>
@@ -3759,13 +3571,12 @@
       <c r="G174" s="114" t="n"/>
       <c r="H174" s="114" t="n"/>
       <c r="I174" s="53" t="n"/>
-      <c r="J174" s="55" t="n"/>
+      <c r="J174" s="74" t="n"/>
       <c r="K174" s="74" t="n"/>
-      <c r="L174" s="74" t="n"/>
-      <c r="M174" s="100" t="n"/>
-      <c r="O174" s="92" t="n"/>
+      <c r="L174" s="100" t="n"/>
+      <c r="N174" s="92" t="n"/>
+      <c r="O174" s="57" t="n"/>
       <c r="P174" s="57" t="n"/>
-      <c r="Q174" s="57" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="74" t="n"/>
@@ -3775,13 +3586,12 @@
       <c r="G175" s="114" t="n"/>
       <c r="H175" s="114" t="n"/>
       <c r="I175" s="53" t="n"/>
-      <c r="J175" s="55" t="n"/>
+      <c r="J175" s="74" t="n"/>
       <c r="K175" s="74" t="n"/>
-      <c r="L175" s="74" t="n"/>
-      <c r="M175" s="100" t="n"/>
-      <c r="O175" s="92" t="n"/>
+      <c r="L175" s="100" t="n"/>
+      <c r="N175" s="92" t="n"/>
+      <c r="O175" s="57" t="n"/>
       <c r="P175" s="57" t="n"/>
-      <c r="Q175" s="57" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="74" t="n"/>
@@ -3792,13 +3602,12 @@
       <c r="G176" s="114" t="n"/>
       <c r="H176" s="114" t="n"/>
       <c r="I176" s="53" t="n"/>
-      <c r="J176" s="55" t="n"/>
+      <c r="J176" s="74" t="n"/>
       <c r="K176" s="74" t="n"/>
-      <c r="L176" s="74" t="n"/>
-      <c r="M176" s="100" t="n"/>
-      <c r="O176" s="92" t="n"/>
+      <c r="L176" s="100" t="n"/>
+      <c r="N176" s="92" t="n"/>
+      <c r="O176" s="57" t="n"/>
       <c r="P176" s="57" t="n"/>
-      <c r="Q176" s="57" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="74" t="n"/>
@@ -3807,13 +3616,12 @@
       <c r="G177" s="114" t="n"/>
       <c r="H177" s="114" t="n"/>
       <c r="I177" s="53" t="n"/>
-      <c r="J177" s="55" t="n"/>
+      <c r="J177" s="74" t="n"/>
       <c r="K177" s="74" t="n"/>
-      <c r="L177" s="74" t="n"/>
-      <c r="M177" s="100" t="n"/>
-      <c r="O177" s="92" t="n"/>
+      <c r="L177" s="100" t="n"/>
+      <c r="N177" s="92" t="n"/>
+      <c r="O177" s="57" t="n"/>
       <c r="P177" s="57" t="n"/>
-      <c r="Q177" s="57" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="74" t="n"/>
@@ -3822,13 +3630,12 @@
       <c r="G178" s="114" t="n"/>
       <c r="H178" s="114" t="n"/>
       <c r="I178" s="53" t="n"/>
-      <c r="J178" s="55" t="n"/>
+      <c r="J178" s="74" t="n"/>
       <c r="K178" s="74" t="n"/>
-      <c r="L178" s="74" t="n"/>
-      <c r="M178" s="100" t="n"/>
-      <c r="O178" s="92" t="n"/>
+      <c r="L178" s="100" t="n"/>
+      <c r="N178" s="92" t="n"/>
+      <c r="O178" s="57" t="n"/>
       <c r="P178" s="57" t="n"/>
-      <c r="Q178" s="57" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="74" t="n"/>
@@ -3836,13 +3643,12 @@
       <c r="G179" s="114" t="n"/>
       <c r="H179" s="114" t="n"/>
       <c r="I179" s="53" t="n"/>
-      <c r="J179" s="55" t="n"/>
+      <c r="J179" s="74" t="n"/>
       <c r="K179" s="74" t="n"/>
-      <c r="L179" s="74" t="n"/>
-      <c r="M179" s="100" t="n"/>
-      <c r="O179" s="92" t="n"/>
+      <c r="L179" s="100" t="n"/>
+      <c r="N179" s="92" t="n"/>
+      <c r="O179" s="57" t="n"/>
       <c r="P179" s="57" t="n"/>
-      <c r="Q179" s="57" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="74" t="n"/>
@@ -3851,91 +3657,84 @@
       <c r="G180" s="114" t="n"/>
       <c r="H180" s="114" t="n"/>
       <c r="I180" s="98" t="n"/>
-      <c r="J180" s="99" t="n"/>
+      <c r="J180" s="74" t="n"/>
       <c r="K180" s="74" t="n"/>
-      <c r="L180" s="74" t="n"/>
-      <c r="M180" s="100" t="n"/>
+      <c r="L180" s="100" t="n"/>
+      <c r="N180" s="57" t="n"/>
       <c r="O180" s="57" t="n"/>
       <c r="P180" s="57" t="n"/>
-      <c r="Q180" s="57" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="74" t="n"/>
       <c r="G181" s="114" t="n"/>
       <c r="H181" s="114" t="n"/>
       <c r="I181" s="98" t="n"/>
-      <c r="J181" s="99" t="n"/>
+      <c r="J181" s="74" t="n"/>
       <c r="K181" s="74" t="n"/>
-      <c r="L181" s="74" t="n"/>
-      <c r="M181" s="100" t="n"/>
+      <c r="L181" s="100" t="n"/>
+      <c r="N181" s="57" t="n"/>
       <c r="O181" s="57" t="n"/>
       <c r="P181" s="57" t="n"/>
-      <c r="Q181" s="57" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="74" t="n"/>
       <c r="G182" s="114" t="n"/>
       <c r="H182" s="114" t="n"/>
       <c r="I182" s="98" t="n"/>
-      <c r="J182" s="99" t="n"/>
+      <c r="J182" s="74" t="n"/>
       <c r="K182" s="74" t="n"/>
-      <c r="L182" s="74" t="n"/>
-      <c r="M182" s="100" t="n"/>
+      <c r="L182" s="100" t="n"/>
+      <c r="N182" s="57" t="n"/>
       <c r="O182" s="57" t="n"/>
       <c r="P182" s="57" t="n"/>
-      <c r="Q182" s="57" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="74" t="n"/>
       <c r="G183" s="114" t="n"/>
       <c r="H183" s="114" t="n"/>
       <c r="I183" s="98" t="n"/>
-      <c r="J183" s="99" t="n"/>
+      <c r="J183" s="74" t="n"/>
       <c r="K183" s="74" t="n"/>
-      <c r="L183" s="74" t="n"/>
-      <c r="M183" s="100" t="n"/>
+      <c r="L183" s="100" t="n"/>
+      <c r="N183" s="57" t="n"/>
       <c r="O183" s="57" t="n"/>
       <c r="P183" s="57" t="n"/>
-      <c r="Q183" s="57" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="74" t="n"/>
       <c r="G184" s="114" t="n"/>
       <c r="H184" s="114" t="n"/>
       <c r="I184" s="98" t="n"/>
-      <c r="J184" s="99" t="n"/>
+      <c r="J184" s="74" t="n"/>
       <c r="K184" s="74" t="n"/>
-      <c r="L184" s="74" t="n"/>
-      <c r="M184" s="100" t="n"/>
+      <c r="L184" s="100" t="n"/>
+      <c r="N184" s="57" t="n"/>
       <c r="O184" s="57" t="n"/>
       <c r="P184" s="57" t="n"/>
-      <c r="Q184" s="57" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="74" t="n"/>
       <c r="G185" s="114" t="n"/>
       <c r="H185" s="114" t="n"/>
       <c r="I185" s="98" t="n"/>
-      <c r="J185" s="99" t="n"/>
+      <c r="J185" s="74" t="n"/>
       <c r="K185" s="74" t="n"/>
-      <c r="L185" s="74" t="n"/>
-      <c r="M185" s="100" t="n"/>
+      <c r="L185" s="100" t="n"/>
+      <c r="N185" s="57" t="n"/>
       <c r="O185" s="57" t="n"/>
       <c r="P185" s="57" t="n"/>
-      <c r="Q185" s="57" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="74" t="n"/>
       <c r="G186" s="114" t="n"/>
       <c r="H186" s="114" t="n"/>
       <c r="I186" s="98" t="n"/>
-      <c r="J186" s="99" t="n"/>
+      <c r="J186" s="74" t="n"/>
       <c r="K186" s="74" t="n"/>
-      <c r="L186" s="74" t="n"/>
-      <c r="M186" s="100" t="n"/>
+      <c r="L186" s="100" t="n"/>
+      <c r="N186" s="57" t="n"/>
       <c r="O186" s="57" t="n"/>
       <c r="P186" s="57" t="n"/>
-      <c r="Q186" s="57" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="74" t="n"/>
@@ -3944,52 +3743,48 @@
       <c r="G187" s="114" t="n"/>
       <c r="H187" s="114" t="n"/>
       <c r="I187" s="98" t="n"/>
-      <c r="J187" s="99" t="n"/>
+      <c r="J187" s="74" t="n"/>
       <c r="K187" s="74" t="n"/>
-      <c r="L187" s="74" t="n"/>
-      <c r="M187" s="100" t="n"/>
+      <c r="L187" s="100" t="n"/>
+      <c r="N187" s="57" t="n"/>
       <c r="O187" s="57" t="n"/>
       <c r="P187" s="57" t="n"/>
-      <c r="Q187" s="57" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="74" t="n"/>
       <c r="G188" s="114" t="n"/>
       <c r="H188" s="114" t="n"/>
       <c r="I188" s="98" t="n"/>
-      <c r="J188" s="99" t="n"/>
+      <c r="J188" s="74" t="n"/>
       <c r="K188" s="74" t="n"/>
-      <c r="L188" s="74" t="n"/>
-      <c r="M188" s="100" t="n"/>
+      <c r="L188" s="100" t="n"/>
+      <c r="N188" s="57" t="n"/>
       <c r="O188" s="57" t="n"/>
       <c r="P188" s="57" t="n"/>
-      <c r="Q188" s="57" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="74" t="n"/>
       <c r="G189" s="114" t="n"/>
       <c r="H189" s="114" t="n"/>
       <c r="I189" s="98" t="n"/>
-      <c r="J189" s="99" t="n"/>
+      <c r="J189" s="74" t="n"/>
       <c r="K189" s="74" t="n"/>
-      <c r="L189" s="74" t="n"/>
-      <c r="M189" s="100" t="n"/>
+      <c r="L189" s="100" t="n"/>
+      <c r="N189" s="57" t="n"/>
       <c r="O189" s="57" t="n"/>
       <c r="P189" s="57" t="n"/>
-      <c r="Q189" s="57" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="74" t="n"/>
       <c r="G190" s="114" t="n"/>
       <c r="H190" s="114" t="n"/>
       <c r="I190" s="98" t="n"/>
-      <c r="J190" s="99" t="n"/>
+      <c r="J190" s="74" t="n"/>
       <c r="K190" s="74" t="n"/>
-      <c r="L190" s="74" t="n"/>
-      <c r="M190" s="100" t="n"/>
+      <c r="L190" s="100" t="n"/>
+      <c r="N190" s="57" t="n"/>
       <c r="O190" s="57" t="n"/>
       <c r="P190" s="57" t="n"/>
-      <c r="Q190" s="57" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="74" t="n"/>
@@ -3997,13 +3792,12 @@
       <c r="G191" s="114" t="n"/>
       <c r="H191" s="114" t="n"/>
       <c r="I191" s="98" t="n"/>
-      <c r="J191" s="99" t="n"/>
+      <c r="J191" s="74" t="n"/>
       <c r="K191" s="74" t="n"/>
-      <c r="L191" s="74" t="n"/>
-      <c r="M191" s="100" t="n"/>
+      <c r="L191" s="100" t="n"/>
+      <c r="N191" s="57" t="n"/>
       <c r="O191" s="57" t="n"/>
       <c r="P191" s="57" t="n"/>
-      <c r="Q191" s="57" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="74" t="n"/>
@@ -4013,13 +3807,12 @@
       <c r="G192" s="114" t="n"/>
       <c r="H192" s="114" t="n"/>
       <c r="I192" s="98" t="n"/>
-      <c r="J192" s="99" t="n"/>
+      <c r="J192" s="74" t="n"/>
       <c r="K192" s="74" t="n"/>
-      <c r="L192" s="74" t="n"/>
-      <c r="M192" s="100" t="n"/>
+      <c r="L192" s="100" t="n"/>
+      <c r="N192" s="57" t="n"/>
       <c r="O192" s="57" t="n"/>
       <c r="P192" s="57" t="n"/>
-      <c r="Q192" s="57" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="74" t="n"/>
@@ -4030,28 +3823,26 @@
       <c r="G193" s="93" t="n"/>
       <c r="H193" s="93" t="n"/>
       <c r="I193" s="98" t="n"/>
-      <c r="J193" s="99" t="n"/>
+      <c r="J193" s="74" t="n"/>
       <c r="K193" s="74" t="n"/>
-      <c r="L193" s="74" t="n"/>
+      <c r="L193" s="100" t="n"/>
       <c r="M193" s="100" t="n"/>
-      <c r="N193" s="100" t="n"/>
+      <c r="N193" s="57" t="n"/>
       <c r="O193" s="57" t="n"/>
       <c r="P193" s="57" t="n"/>
-      <c r="Q193" s="57" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="74" t="n"/>
       <c r="G194" s="93" t="n"/>
       <c r="H194" s="93" t="n"/>
       <c r="I194" s="98" t="n"/>
-      <c r="J194" s="99" t="n"/>
+      <c r="J194" s="74" t="n"/>
       <c r="K194" s="74" t="n"/>
-      <c r="L194" s="74" t="n"/>
+      <c r="L194" s="100" t="n"/>
       <c r="M194" s="100" t="n"/>
-      <c r="N194" s="100" t="n"/>
+      <c r="N194" s="57" t="n"/>
       <c r="O194" s="57" t="n"/>
       <c r="P194" s="57" t="n"/>
-      <c r="Q194" s="57" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="74" t="n"/>
@@ -4062,156 +3853,144 @@
       <c r="G195" s="93" t="n"/>
       <c r="H195" s="93" t="n"/>
       <c r="I195" s="98" t="n"/>
-      <c r="J195" s="99" t="n"/>
+      <c r="J195" s="74" t="n"/>
       <c r="K195" s="74" t="n"/>
-      <c r="L195" s="74" t="n"/>
-      <c r="M195" s="100" t="n"/>
+      <c r="L195" s="100" t="n"/>
+      <c r="N195" s="57" t="n"/>
       <c r="O195" s="57" t="n"/>
       <c r="P195" s="57" t="n"/>
-      <c r="Q195" s="57" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="74" t="n"/>
       <c r="G196" s="93" t="n"/>
       <c r="H196" s="93" t="n"/>
       <c r="I196" s="98" t="n"/>
-      <c r="J196" s="99" t="n"/>
+      <c r="J196" s="74" t="n"/>
       <c r="K196" s="74" t="n"/>
-      <c r="L196" s="74" t="n"/>
-      <c r="M196" s="100" t="n"/>
+      <c r="L196" s="100" t="n"/>
+      <c r="N196" s="57" t="n"/>
       <c r="O196" s="57" t="n"/>
       <c r="P196" s="57" t="n"/>
-      <c r="Q196" s="57" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="74" t="n"/>
       <c r="G197" s="93" t="n"/>
       <c r="H197" s="93" t="n"/>
       <c r="I197" s="98" t="n"/>
-      <c r="J197" s="99" t="n"/>
+      <c r="J197" s="74" t="n"/>
       <c r="K197" s="74" t="n"/>
-      <c r="L197" s="74" t="n"/>
-      <c r="M197" s="100" t="n"/>
+      <c r="L197" s="100" t="n"/>
+      <c r="N197" s="57" t="n"/>
       <c r="O197" s="57" t="n"/>
       <c r="P197" s="57" t="n"/>
-      <c r="Q197" s="57" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="74" t="n"/>
       <c r="G198" s="93" t="n"/>
       <c r="H198" s="93" t="n"/>
       <c r="I198" s="98" t="n"/>
-      <c r="J198" s="99" t="n"/>
+      <c r="J198" s="74" t="n"/>
       <c r="K198" s="74" t="n"/>
-      <c r="L198" s="74" t="n"/>
-      <c r="M198" s="100" t="n"/>
+      <c r="L198" s="100" t="n"/>
+      <c r="N198" s="57" t="n"/>
       <c r="O198" s="57" t="n"/>
       <c r="P198" s="57" t="n"/>
-      <c r="Q198" s="57" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="74" t="n"/>
       <c r="G199" s="93" t="n"/>
       <c r="H199" s="93" t="n"/>
       <c r="I199" s="98" t="n"/>
-      <c r="J199" s="99" t="n"/>
+      <c r="J199" s="74" t="n"/>
       <c r="K199" s="74" t="n"/>
-      <c r="L199" s="74" t="n"/>
-      <c r="M199" s="100" t="n"/>
+      <c r="L199" s="100" t="n"/>
+      <c r="N199" s="57" t="n"/>
       <c r="O199" s="57" t="n"/>
       <c r="P199" s="57" t="n"/>
-      <c r="Q199" s="57" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="74" t="n"/>
       <c r="G200" s="93" t="n"/>
       <c r="H200" s="93" t="n"/>
       <c r="I200" s="98" t="n"/>
-      <c r="J200" s="99" t="n"/>
+      <c r="J200" s="74" t="n"/>
       <c r="K200" s="74" t="n"/>
-      <c r="L200" s="74" t="n"/>
-      <c r="M200" s="100" t="n"/>
+      <c r="L200" s="100" t="n"/>
+      <c r="N200" s="57" t="n"/>
       <c r="O200" s="57" t="n"/>
       <c r="P200" s="57" t="n"/>
-      <c r="Q200" s="57" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="74" t="n"/>
       <c r="G201" s="93" t="n"/>
       <c r="H201" s="93" t="n"/>
       <c r="I201" s="98" t="n"/>
-      <c r="J201" s="99" t="n"/>
+      <c r="J201" s="74" t="n"/>
       <c r="K201" s="74" t="n"/>
-      <c r="L201" s="74" t="n"/>
-      <c r="M201" s="100" t="n"/>
+      <c r="L201" s="100" t="n"/>
+      <c r="N201" s="57" t="n"/>
       <c r="O201" s="57" t="n"/>
       <c r="P201" s="57" t="n"/>
-      <c r="Q201" s="57" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="74" t="n"/>
       <c r="G202" s="93" t="n"/>
       <c r="H202" s="93" t="n"/>
       <c r="I202" s="98" t="n"/>
-      <c r="J202" s="99" t="n"/>
+      <c r="J202" s="74" t="n"/>
       <c r="K202" s="74" t="n"/>
-      <c r="L202" s="74" t="n"/>
-      <c r="M202" s="100" t="n"/>
+      <c r="L202" s="100" t="n"/>
+      <c r="N202" s="57" t="n"/>
       <c r="O202" s="57" t="n"/>
       <c r="P202" s="57" t="n"/>
-      <c r="Q202" s="57" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="74" t="n"/>
       <c r="G203" s="93" t="n"/>
       <c r="H203" s="93" t="n"/>
       <c r="I203" s="98" t="n"/>
-      <c r="J203" s="99" t="n"/>
+      <c r="J203" s="74" t="n"/>
       <c r="K203" s="74" t="n"/>
-      <c r="L203" s="74" t="n"/>
-      <c r="M203" s="100" t="n"/>
+      <c r="L203" s="100" t="n"/>
+      <c r="N203" s="57" t="n"/>
       <c r="O203" s="57" t="n"/>
       <c r="P203" s="57" t="n"/>
-      <c r="Q203" s="57" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="74" t="n"/>
       <c r="G204" s="93" t="n"/>
       <c r="H204" s="93" t="n"/>
       <c r="I204" s="98" t="n"/>
-      <c r="J204" s="99" t="n"/>
+      <c r="J204" s="74" t="n"/>
       <c r="K204" s="74" t="n"/>
-      <c r="L204" s="74" t="n"/>
-      <c r="M204" s="100" t="n"/>
+      <c r="L204" s="100" t="n"/>
+      <c r="N204" s="57" t="n"/>
       <c r="O204" s="57" t="n"/>
       <c r="P204" s="57" t="n"/>
-      <c r="Q204" s="57" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="74" t="n"/>
       <c r="G205" s="93" t="n"/>
       <c r="H205" s="93" t="n"/>
       <c r="I205" s="98" t="n"/>
-      <c r="J205" s="99" t="n"/>
+      <c r="J205" s="74" t="n"/>
       <c r="K205" s="74" t="n"/>
-      <c r="L205" s="74" t="n"/>
-      <c r="M205" s="100" t="n"/>
+      <c r="L205" s="100" t="n"/>
+      <c r="N205" s="57" t="n"/>
       <c r="O205" s="57" t="n"/>
       <c r="P205" s="57" t="n"/>
-      <c r="Q205" s="57" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="74" t="n"/>
       <c r="G206" s="93" t="n"/>
       <c r="H206" s="93" t="n"/>
       <c r="I206" s="98" t="n"/>
-      <c r="J206" s="99" t="n"/>
+      <c r="J206" s="74" t="n"/>
       <c r="K206" s="74" t="n"/>
-      <c r="L206" s="74" t="n"/>
-      <c r="M206" s="100" t="n"/>
+      <c r="L206" s="100" t="n"/>
+      <c r="N206" s="57" t="n"/>
       <c r="O206" s="57" t="n"/>
       <c r="P206" s="57" t="n"/>
-      <c r="Q206" s="57" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="74" t="n"/>
@@ -4223,26 +4002,24 @@
       <c r="G207" s="107" t="n"/>
       <c r="H207" s="107" t="n"/>
       <c r="I207" s="98" t="n"/>
-      <c r="J207" s="99" t="n"/>
+      <c r="J207" s="74" t="n"/>
       <c r="K207" s="74" t="n"/>
-      <c r="L207" s="74" t="n"/>
-      <c r="M207" s="100" t="n"/>
+      <c r="L207" s="100" t="n"/>
+      <c r="N207" s="57" t="n"/>
       <c r="O207" s="57" t="n"/>
       <c r="P207" s="57" t="n"/>
-      <c r="Q207" s="57" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="74" t="n"/>
       <c r="G208" s="107" t="n"/>
       <c r="H208" s="107" t="n"/>
       <c r="I208" s="98" t="n"/>
-      <c r="J208" s="99" t="n"/>
+      <c r="J208" s="74" t="n"/>
       <c r="K208" s="74" t="n"/>
-      <c r="L208" s="74" t="n"/>
-      <c r="M208" s="100" t="n"/>
+      <c r="L208" s="100" t="n"/>
+      <c r="N208" s="57" t="n"/>
       <c r="O208" s="57" t="n"/>
       <c r="P208" s="57" t="n"/>
-      <c r="Q208" s="57" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="74" t="n"/>
@@ -4251,52 +4028,48 @@
       <c r="G209" s="107" t="n"/>
       <c r="H209" s="107" t="n"/>
       <c r="I209" s="98" t="n"/>
-      <c r="J209" s="99" t="n"/>
+      <c r="J209" s="74" t="n"/>
       <c r="K209" s="74" t="n"/>
-      <c r="L209" s="74" t="n"/>
-      <c r="M209" s="100" t="n"/>
+      <c r="L209" s="100" t="n"/>
+      <c r="N209" s="57" t="n"/>
       <c r="O209" s="57" t="n"/>
       <c r="P209" s="57" t="n"/>
-      <c r="Q209" s="57" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="74" t="n"/>
       <c r="G210" s="107" t="n"/>
       <c r="H210" s="107" t="n"/>
       <c r="I210" s="98" t="n"/>
-      <c r="J210" s="99" t="n"/>
+      <c r="J210" s="74" t="n"/>
       <c r="K210" s="74" t="n"/>
-      <c r="L210" s="74" t="n"/>
-      <c r="M210" s="100" t="n"/>
+      <c r="L210" s="100" t="n"/>
+      <c r="N210" s="57" t="n"/>
       <c r="O210" s="57" t="n"/>
       <c r="P210" s="57" t="n"/>
-      <c r="Q210" s="57" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="74" t="n"/>
       <c r="G211" s="107" t="n"/>
       <c r="H211" s="107" t="n"/>
       <c r="I211" s="98" t="n"/>
-      <c r="J211" s="99" t="n"/>
+      <c r="J211" s="74" t="n"/>
       <c r="K211" s="74" t="n"/>
-      <c r="L211" s="74" t="n"/>
-      <c r="M211" s="100" t="n"/>
+      <c r="L211" s="100" t="n"/>
+      <c r="N211" s="57" t="n"/>
       <c r="O211" s="57" t="n"/>
       <c r="P211" s="57" t="n"/>
-      <c r="Q211" s="57" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="74" t="n"/>
       <c r="G212" s="107" t="n"/>
       <c r="H212" s="107" t="n"/>
       <c r="I212" s="98" t="n"/>
-      <c r="J212" s="99" t="n"/>
+      <c r="J212" s="74" t="n"/>
       <c r="K212" s="74" t="n"/>
-      <c r="L212" s="74" t="n"/>
-      <c r="M212" s="100" t="n"/>
+      <c r="L212" s="100" t="n"/>
+      <c r="N212" s="57" t="n"/>
       <c r="O212" s="57" t="n"/>
       <c r="P212" s="57" t="n"/>
-      <c r="Q212" s="57" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="74" t="n"/>
@@ -4304,13 +4077,12 @@
       <c r="G213" s="107" t="n"/>
       <c r="H213" s="107" t="n"/>
       <c r="I213" s="98" t="n"/>
-      <c r="J213" s="99" t="n"/>
+      <c r="J213" s="74" t="n"/>
       <c r="K213" s="74" t="n"/>
-      <c r="L213" s="74" t="n"/>
-      <c r="M213" s="100" t="n"/>
+      <c r="L213" s="100" t="n"/>
+      <c r="N213" s="57" t="n"/>
       <c r="O213" s="57" t="n"/>
       <c r="P213" s="57" t="n"/>
-      <c r="Q213" s="57" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="74" t="n"/>
@@ -4318,13 +4090,12 @@
       <c r="G214" s="107" t="n"/>
       <c r="H214" s="107" t="n"/>
       <c r="I214" s="98" t="n"/>
-      <c r="J214" s="99" t="n"/>
+      <c r="J214" s="74" t="n"/>
       <c r="K214" s="74" t="n"/>
-      <c r="L214" s="74" t="n"/>
-      <c r="M214" s="100" t="n"/>
+      <c r="L214" s="100" t="n"/>
+      <c r="N214" s="57" t="n"/>
       <c r="O214" s="57" t="n"/>
       <c r="P214" s="57" t="n"/>
-      <c r="Q214" s="57" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="74" t="n"/>
@@ -4332,13 +4103,12 @@
       <c r="G215" s="107" t="n"/>
       <c r="H215" s="107" t="n"/>
       <c r="I215" s="98" t="n"/>
-      <c r="J215" s="99" t="n"/>
+      <c r="J215" s="74" t="n"/>
       <c r="K215" s="74" t="n"/>
-      <c r="L215" s="74" t="n"/>
-      <c r="M215" s="100" t="n"/>
+      <c r="L215" s="100" t="n"/>
+      <c r="N215" s="57" t="n"/>
       <c r="O215" s="57" t="n"/>
       <c r="P215" s="57" t="n"/>
-      <c r="Q215" s="57" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="74" t="n"/>
@@ -4346,65 +4116,60 @@
       <c r="G216" s="107" t="n"/>
       <c r="H216" s="107" t="n"/>
       <c r="I216" s="98" t="n"/>
-      <c r="J216" s="99" t="n"/>
+      <c r="J216" s="74" t="n"/>
       <c r="K216" s="74" t="n"/>
-      <c r="L216" s="74" t="n"/>
-      <c r="M216" s="100" t="n"/>
+      <c r="L216" s="100" t="n"/>
+      <c r="N216" s="57" t="n"/>
       <c r="O216" s="57" t="n"/>
       <c r="P216" s="57" t="n"/>
-      <c r="Q216" s="57" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="74" t="n"/>
       <c r="G217" s="107" t="n"/>
       <c r="H217" s="107" t="n"/>
       <c r="I217" s="98" t="n"/>
-      <c r="J217" s="99" t="n"/>
+      <c r="J217" s="74" t="n"/>
       <c r="K217" s="74" t="n"/>
-      <c r="L217" s="74" t="n"/>
-      <c r="M217" s="100" t="n"/>
+      <c r="L217" s="100" t="n"/>
+      <c r="N217" s="57" t="n"/>
       <c r="O217" s="57" t="n"/>
       <c r="P217" s="57" t="n"/>
-      <c r="Q217" s="57" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="74" t="n"/>
       <c r="G218" s="107" t="n"/>
       <c r="H218" s="107" t="n"/>
       <c r="I218" s="98" t="n"/>
-      <c r="J218" s="99" t="n"/>
+      <c r="J218" s="74" t="n"/>
       <c r="K218" s="74" t="n"/>
-      <c r="L218" s="74" t="n"/>
-      <c r="M218" s="100" t="n"/>
+      <c r="L218" s="100" t="n"/>
+      <c r="N218" s="57" t="n"/>
       <c r="O218" s="57" t="n"/>
       <c r="P218" s="57" t="n"/>
-      <c r="Q218" s="57" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="74" t="n"/>
       <c r="G219" s="107" t="n"/>
       <c r="H219" s="107" t="n"/>
       <c r="I219" s="98" t="n"/>
-      <c r="J219" s="99" t="n"/>
+      <c r="J219" s="74" t="n"/>
       <c r="K219" s="74" t="n"/>
-      <c r="L219" s="74" t="n"/>
-      <c r="M219" s="100" t="n"/>
+      <c r="L219" s="100" t="n"/>
+      <c r="N219" s="57" t="n"/>
       <c r="O219" s="57" t="n"/>
       <c r="P219" s="57" t="n"/>
-      <c r="Q219" s="57" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="74" t="n"/>
       <c r="G220" s="107" t="n"/>
       <c r="H220" s="107" t="n"/>
       <c r="I220" s="98" t="n"/>
-      <c r="J220" s="99" t="n"/>
+      <c r="J220" s="74" t="n"/>
       <c r="K220" s="74" t="n"/>
-      <c r="L220" s="74" t="n"/>
-      <c r="M220" s="100" t="n"/>
+      <c r="L220" s="100" t="n"/>
+      <c r="N220" s="57" t="n"/>
       <c r="O220" s="57" t="n"/>
       <c r="P220" s="57" t="n"/>
-      <c r="Q220" s="57" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="74" t="n"/>
@@ -4413,13 +4178,12 @@
       <c r="G221" s="107" t="n"/>
       <c r="H221" s="107" t="n"/>
       <c r="I221" s="98" t="n"/>
-      <c r="J221" s="99" t="n"/>
+      <c r="J221" s="74" t="n"/>
       <c r="K221" s="74" t="n"/>
-      <c r="L221" s="74" t="n"/>
-      <c r="M221" s="100" t="n"/>
+      <c r="L221" s="100" t="n"/>
+      <c r="N221" s="57" t="n"/>
       <c r="O221" s="57" t="n"/>
       <c r="P221" s="57" t="n"/>
-      <c r="Q221" s="57" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="74" t="n"/>
@@ -4427,52 +4191,48 @@
       <c r="G222" s="107" t="n"/>
       <c r="H222" s="107" t="n"/>
       <c r="I222" s="98" t="n"/>
-      <c r="J222" s="99" t="n"/>
+      <c r="J222" s="74" t="n"/>
       <c r="K222" s="74" t="n"/>
-      <c r="L222" s="74" t="n"/>
-      <c r="M222" s="100" t="n"/>
+      <c r="L222" s="100" t="n"/>
+      <c r="N222" s="57" t="n"/>
       <c r="O222" s="57" t="n"/>
       <c r="P222" s="57" t="n"/>
-      <c r="Q222" s="57" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="74" t="n"/>
       <c r="G223" s="107" t="n"/>
       <c r="H223" s="107" t="n"/>
       <c r="I223" s="98" t="n"/>
-      <c r="J223" s="99" t="n"/>
+      <c r="J223" s="74" t="n"/>
       <c r="K223" s="74" t="n"/>
-      <c r="L223" s="74" t="n"/>
-      <c r="M223" s="100" t="n"/>
+      <c r="L223" s="100" t="n"/>
+      <c r="N223" s="57" t="n"/>
       <c r="O223" s="57" t="n"/>
       <c r="P223" s="57" t="n"/>
-      <c r="Q223" s="57" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="74" t="n"/>
       <c r="G224" s="107" t="n"/>
       <c r="H224" s="107" t="n"/>
       <c r="I224" s="98" t="n"/>
-      <c r="J224" s="99" t="n"/>
+      <c r="J224" s="74" t="n"/>
       <c r="K224" s="74" t="n"/>
-      <c r="L224" s="74" t="n"/>
-      <c r="M224" s="100" t="n"/>
+      <c r="L224" s="100" t="n"/>
+      <c r="N224" s="57" t="n"/>
       <c r="O224" s="57" t="n"/>
       <c r="P224" s="57" t="n"/>
-      <c r="Q224" s="57" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="74" t="n"/>
       <c r="G225" s="107" t="n"/>
       <c r="H225" s="107" t="n"/>
       <c r="I225" s="98" t="n"/>
-      <c r="J225" s="99" t="n"/>
+      <c r="J225" s="74" t="n"/>
       <c r="K225" s="74" t="n"/>
-      <c r="L225" s="74" t="n"/>
-      <c r="M225" s="100" t="n"/>
+      <c r="L225" s="100" t="n"/>
+      <c r="N225" s="57" t="n"/>
       <c r="O225" s="57" t="n"/>
       <c r="P225" s="57" t="n"/>
-      <c r="Q225" s="57" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="74" t="n"/>
@@ -4480,52 +4240,48 @@
       <c r="G226" s="107" t="n"/>
       <c r="H226" s="107" t="n"/>
       <c r="I226" s="98" t="n"/>
-      <c r="J226" s="99" t="n"/>
+      <c r="J226" s="74" t="n"/>
       <c r="K226" s="74" t="n"/>
-      <c r="L226" s="74" t="n"/>
-      <c r="M226" s="100" t="n"/>
+      <c r="L226" s="100" t="n"/>
+      <c r="N226" s="57" t="n"/>
       <c r="O226" s="57" t="n"/>
       <c r="P226" s="57" t="n"/>
-      <c r="Q226" s="57" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="74" t="n"/>
       <c r="G227" s="107" t="n"/>
       <c r="H227" s="107" t="n"/>
       <c r="I227" s="98" t="n"/>
-      <c r="J227" s="99" t="n"/>
+      <c r="J227" s="74" t="n"/>
       <c r="K227" s="74" t="n"/>
-      <c r="L227" s="74" t="n"/>
-      <c r="M227" s="100" t="n"/>
+      <c r="L227" s="100" t="n"/>
+      <c r="N227" s="57" t="n"/>
       <c r="O227" s="57" t="n"/>
       <c r="P227" s="57" t="n"/>
-      <c r="Q227" s="57" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="74" t="n"/>
       <c r="G228" s="107" t="n"/>
       <c r="H228" s="107" t="n"/>
       <c r="I228" s="98" t="n"/>
-      <c r="J228" s="99" t="n"/>
+      <c r="J228" s="74" t="n"/>
       <c r="K228" s="74" t="n"/>
-      <c r="L228" s="74" t="n"/>
-      <c r="M228" s="100" t="n"/>
+      <c r="L228" s="100" t="n"/>
+      <c r="N228" s="57" t="n"/>
       <c r="O228" s="57" t="n"/>
       <c r="P228" s="57" t="n"/>
-      <c r="Q228" s="57" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="74" t="n"/>
       <c r="G229" s="107" t="n"/>
       <c r="H229" s="107" t="n"/>
       <c r="I229" s="98" t="n"/>
-      <c r="J229" s="99" t="n"/>
+      <c r="J229" s="74" t="n"/>
       <c r="K229" s="74" t="n"/>
-      <c r="L229" s="74" t="n"/>
-      <c r="M229" s="100" t="n"/>
+      <c r="L229" s="100" t="n"/>
+      <c r="N229" s="57" t="n"/>
       <c r="O229" s="57" t="n"/>
       <c r="P229" s="57" t="n"/>
-      <c r="Q229" s="57" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="74" t="n"/>
@@ -4534,13 +4290,12 @@
       <c r="G230" s="107" t="n"/>
       <c r="H230" s="107" t="n"/>
       <c r="I230" s="98" t="n"/>
-      <c r="J230" s="99" t="n"/>
+      <c r="J230" s="74" t="n"/>
       <c r="K230" s="74" t="n"/>
-      <c r="L230" s="74" t="n"/>
-      <c r="M230" s="100" t="n"/>
+      <c r="L230" s="100" t="n"/>
+      <c r="N230" s="57" t="n"/>
       <c r="O230" s="57" t="n"/>
       <c r="P230" s="57" t="n"/>
-      <c r="Q230" s="57" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="74" t="n"/>
@@ -4548,52 +4303,48 @@
       <c r="G231" s="107" t="n"/>
       <c r="H231" s="107" t="n"/>
       <c r="I231" s="98" t="n"/>
-      <c r="J231" s="99" t="n"/>
+      <c r="J231" s="74" t="n"/>
       <c r="K231" s="74" t="n"/>
-      <c r="L231" s="74" t="n"/>
-      <c r="M231" s="100" t="n"/>
+      <c r="L231" s="100" t="n"/>
+      <c r="N231" s="57" t="n"/>
       <c r="O231" s="57" t="n"/>
       <c r="P231" s="57" t="n"/>
-      <c r="Q231" s="57" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="74" t="n"/>
       <c r="G232" s="107" t="n"/>
       <c r="H232" s="107" t="n"/>
       <c r="I232" s="98" t="n"/>
-      <c r="J232" s="99" t="n"/>
+      <c r="J232" s="74" t="n"/>
       <c r="K232" s="74" t="n"/>
-      <c r="L232" s="74" t="n"/>
-      <c r="M232" s="100" t="n"/>
+      <c r="L232" s="100" t="n"/>
+      <c r="N232" s="57" t="n"/>
       <c r="O232" s="57" t="n"/>
       <c r="P232" s="57" t="n"/>
-      <c r="Q232" s="57" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="74" t="n"/>
       <c r="G233" s="107" t="n"/>
       <c r="H233" s="107" t="n"/>
       <c r="I233" s="98" t="n"/>
-      <c r="J233" s="99" t="n"/>
+      <c r="J233" s="74" t="n"/>
       <c r="K233" s="74" t="n"/>
-      <c r="L233" s="74" t="n"/>
-      <c r="M233" s="100" t="n"/>
+      <c r="L233" s="100" t="n"/>
+      <c r="N233" s="57" t="n"/>
       <c r="O233" s="57" t="n"/>
       <c r="P233" s="57" t="n"/>
-      <c r="Q233" s="57" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="74" t="n"/>
       <c r="G234" s="107" t="n"/>
       <c r="H234" s="107" t="n"/>
       <c r="I234" s="98" t="n"/>
-      <c r="J234" s="99" t="n"/>
+      <c r="J234" s="74" t="n"/>
       <c r="K234" s="74" t="n"/>
-      <c r="L234" s="74" t="n"/>
-      <c r="M234" s="100" t="n"/>
+      <c r="L234" s="100" t="n"/>
+      <c r="N234" s="57" t="n"/>
       <c r="O234" s="57" t="n"/>
       <c r="P234" s="57" t="n"/>
-      <c r="Q234" s="57" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="74" t="n"/>
@@ -4601,52 +4352,48 @@
       <c r="G235" s="107" t="n"/>
       <c r="H235" s="107" t="n"/>
       <c r="I235" s="98" t="n"/>
-      <c r="J235" s="99" t="n"/>
+      <c r="J235" s="74" t="n"/>
       <c r="K235" s="74" t="n"/>
-      <c r="L235" s="74" t="n"/>
-      <c r="M235" s="100" t="n"/>
+      <c r="L235" s="100" t="n"/>
+      <c r="N235" s="57" t="n"/>
       <c r="O235" s="57" t="n"/>
       <c r="P235" s="57" t="n"/>
-      <c r="Q235" s="57" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="74" t="n"/>
       <c r="G236" s="107" t="n"/>
       <c r="H236" s="107" t="n"/>
       <c r="I236" s="98" t="n"/>
-      <c r="J236" s="99" t="n"/>
+      <c r="J236" s="74" t="n"/>
       <c r="K236" s="74" t="n"/>
-      <c r="L236" s="74" t="n"/>
-      <c r="M236" s="100" t="n"/>
+      <c r="L236" s="100" t="n"/>
+      <c r="N236" s="57" t="n"/>
       <c r="O236" s="57" t="n"/>
       <c r="P236" s="57" t="n"/>
-      <c r="Q236" s="57" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="74" t="n"/>
       <c r="G237" s="107" t="n"/>
       <c r="H237" s="107" t="n"/>
       <c r="I237" s="98" t="n"/>
-      <c r="J237" s="99" t="n"/>
+      <c r="J237" s="74" t="n"/>
       <c r="K237" s="74" t="n"/>
-      <c r="L237" s="74" t="n"/>
-      <c r="M237" s="100" t="n"/>
+      <c r="L237" s="100" t="n"/>
+      <c r="N237" s="57" t="n"/>
       <c r="O237" s="57" t="n"/>
       <c r="P237" s="57" t="n"/>
-      <c r="Q237" s="57" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="74" t="n"/>
       <c r="G238" s="107" t="n"/>
       <c r="H238" s="107" t="n"/>
       <c r="I238" s="98" t="n"/>
-      <c r="J238" s="99" t="n"/>
+      <c r="J238" s="74" t="n"/>
       <c r="K238" s="74" t="n"/>
-      <c r="L238" s="74" t="n"/>
-      <c r="M238" s="100" t="n"/>
+      <c r="L238" s="100" t="n"/>
+      <c r="N238" s="57" t="n"/>
       <c r="O238" s="57" t="n"/>
       <c r="P238" s="57" t="n"/>
-      <c r="Q238" s="57" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="88" t="n"/>
@@ -4658,14 +4405,13 @@
       <c r="G239" s="88" t="n"/>
       <c r="H239" s="88" t="n"/>
       <c r="I239" s="88" t="n"/>
-      <c r="J239" s="112" t="n"/>
+      <c r="J239" s="88" t="n"/>
       <c r="K239" s="88" t="n"/>
       <c r="L239" s="88" t="n"/>
       <c r="M239" s="88" t="n"/>
-      <c r="N239" s="88" t="n"/>
+      <c r="N239" s="57" t="n"/>
       <c r="O239" s="57" t="n"/>
       <c r="P239" s="57" t="n"/>
-      <c r="Q239" s="57" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="88" t="n"/>
@@ -4677,14 +4423,13 @@
       <c r="G240" s="88" t="n"/>
       <c r="H240" s="88" t="n"/>
       <c r="I240" s="88" t="n"/>
-      <c r="J240" s="112" t="n"/>
+      <c r="J240" s="88" t="n"/>
       <c r="K240" s="88" t="n"/>
       <c r="L240" s="88" t="n"/>
       <c r="M240" s="88" t="n"/>
-      <c r="N240" s="88" t="n"/>
+      <c r="N240" s="57" t="n"/>
       <c r="O240" s="57" t="n"/>
       <c r="P240" s="57" t="n"/>
-      <c r="Q240" s="57" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="88" t="n"/>
@@ -4696,14 +4441,13 @@
       <c r="G241" s="88" t="n"/>
       <c r="H241" s="88" t="n"/>
       <c r="I241" s="88" t="n"/>
-      <c r="J241" s="112" t="n"/>
+      <c r="J241" s="88" t="n"/>
       <c r="K241" s="88" t="n"/>
       <c r="L241" s="88" t="n"/>
       <c r="M241" s="88" t="n"/>
-      <c r="N241" s="88" t="n"/>
+      <c r="N241" s="57" t="n"/>
       <c r="O241" s="57" t="n"/>
       <c r="P241" s="57" t="n"/>
-      <c r="Q241" s="57" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="88" t="n"/>
@@ -4715,14 +4459,13 @@
       <c r="G242" s="88" t="n"/>
       <c r="H242" s="88" t="n"/>
       <c r="I242" s="88" t="n"/>
-      <c r="J242" s="112" t="n"/>
+      <c r="J242" s="88" t="n"/>
       <c r="K242" s="88" t="n"/>
       <c r="L242" s="88" t="n"/>
       <c r="M242" s="88" t="n"/>
-      <c r="N242" s="88" t="n"/>
+      <c r="N242" s="57" t="n"/>
       <c r="O242" s="57" t="n"/>
       <c r="P242" s="57" t="n"/>
-      <c r="Q242" s="57" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="88" t="n"/>
@@ -4734,14 +4477,13 @@
       <c r="G243" s="88" t="n"/>
       <c r="H243" s="88" t="n"/>
       <c r="I243" s="88" t="n"/>
-      <c r="J243" s="112" t="n"/>
+      <c r="J243" s="88" t="n"/>
       <c r="K243" s="88" t="n"/>
       <c r="L243" s="88" t="n"/>
       <c r="M243" s="88" t="n"/>
-      <c r="N243" s="88" t="n"/>
+      <c r="N243" s="57" t="n"/>
       <c r="O243" s="57" t="n"/>
       <c r="P243" s="57" t="n"/>
-      <c r="Q243" s="57" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="88" t="n"/>
@@ -4753,14 +4495,13 @@
       <c r="G244" s="88" t="n"/>
       <c r="H244" s="88" t="n"/>
       <c r="I244" s="88" t="n"/>
-      <c r="J244" s="112" t="n"/>
+      <c r="J244" s="88" t="n"/>
       <c r="K244" s="88" t="n"/>
       <c r="L244" s="88" t="n"/>
       <c r="M244" s="88" t="n"/>
-      <c r="N244" s="88" t="n"/>
+      <c r="N244" s="57" t="n"/>
       <c r="O244" s="57" t="n"/>
       <c r="P244" s="57" t="n"/>
-      <c r="Q244" s="57" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="88" t="n"/>
@@ -4772,14 +4513,13 @@
       <c r="G245" s="88" t="n"/>
       <c r="H245" s="88" t="n"/>
       <c r="I245" s="88" t="n"/>
-      <c r="J245" s="112" t="n"/>
+      <c r="J245" s="88" t="n"/>
       <c r="K245" s="88" t="n"/>
       <c r="L245" s="88" t="n"/>
       <c r="M245" s="88" t="n"/>
-      <c r="N245" s="88" t="n"/>
+      <c r="N245" s="57" t="n"/>
       <c r="O245" s="57" t="n"/>
       <c r="P245" s="57" t="n"/>
-      <c r="Q245" s="57" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="88" t="n"/>
@@ -4791,14 +4531,13 @@
       <c r="G246" s="88" t="n"/>
       <c r="H246" s="88" t="n"/>
       <c r="I246" s="88" t="n"/>
-      <c r="J246" s="112" t="n"/>
+      <c r="J246" s="88" t="n"/>
       <c r="K246" s="88" t="n"/>
       <c r="L246" s="88" t="n"/>
       <c r="M246" s="88" t="n"/>
-      <c r="N246" s="88" t="n"/>
+      <c r="N246" s="57" t="n"/>
       <c r="O246" s="57" t="n"/>
       <c r="P246" s="57" t="n"/>
-      <c r="Q246" s="57" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="88" t="n"/>
@@ -4810,14 +4549,13 @@
       <c r="G247" s="88" t="n"/>
       <c r="H247" s="88" t="n"/>
       <c r="I247" s="88" t="n"/>
-      <c r="J247" s="112" t="n"/>
+      <c r="J247" s="88" t="n"/>
       <c r="K247" s="88" t="n"/>
       <c r="L247" s="88" t="n"/>
       <c r="M247" s="88" t="n"/>
-      <c r="N247" s="88" t="n"/>
+      <c r="N247" s="57" t="n"/>
       <c r="O247" s="57" t="n"/>
       <c r="P247" s="57" t="n"/>
-      <c r="Q247" s="57" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="88" t="n"/>
@@ -4829,14 +4567,13 @@
       <c r="G248" s="88" t="n"/>
       <c r="H248" s="88" t="n"/>
       <c r="I248" s="88" t="n"/>
-      <c r="J248" s="112" t="n"/>
+      <c r="J248" s="88" t="n"/>
       <c r="K248" s="88" t="n"/>
       <c r="L248" s="88" t="n"/>
       <c r="M248" s="88" t="n"/>
-      <c r="N248" s="88" t="n"/>
+      <c r="N248" s="57" t="n"/>
       <c r="O248" s="57" t="n"/>
       <c r="P248" s="57" t="n"/>
-      <c r="Q248" s="57" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="88" t="n"/>
@@ -4848,14 +4585,13 @@
       <c r="G249" s="88" t="n"/>
       <c r="H249" s="88" t="n"/>
       <c r="I249" s="88" t="n"/>
-      <c r="J249" s="112" t="n"/>
+      <c r="J249" s="88" t="n"/>
       <c r="K249" s="88" t="n"/>
       <c r="L249" s="88" t="n"/>
       <c r="M249" s="88" t="n"/>
-      <c r="N249" s="88" t="n"/>
+      <c r="N249" s="57" t="n"/>
       <c r="O249" s="57" t="n"/>
       <c r="P249" s="57" t="n"/>
-      <c r="Q249" s="57" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="88" t="n"/>
@@ -4867,14 +4603,13 @@
       <c r="G250" s="88" t="n"/>
       <c r="H250" s="88" t="n"/>
       <c r="I250" s="88" t="n"/>
-      <c r="J250" s="112" t="n"/>
+      <c r="J250" s="88" t="n"/>
       <c r="K250" s="88" t="n"/>
       <c r="L250" s="88" t="n"/>
       <c r="M250" s="88" t="n"/>
-      <c r="N250" s="88" t="n"/>
+      <c r="N250" s="57" t="n"/>
       <c r="O250" s="57" t="n"/>
       <c r="P250" s="57" t="n"/>
-      <c r="Q250" s="57" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="88" t="n"/>
@@ -4886,14 +4621,13 @@
       <c r="G251" s="88" t="n"/>
       <c r="H251" s="88" t="n"/>
       <c r="I251" s="88" t="n"/>
-      <c r="J251" s="112" t="n"/>
+      <c r="J251" s="88" t="n"/>
       <c r="K251" s="88" t="n"/>
       <c r="L251" s="88" t="n"/>
       <c r="M251" s="88" t="n"/>
-      <c r="N251" s="88" t="n"/>
+      <c r="N251" s="57" t="n"/>
       <c r="O251" s="57" t="n"/>
       <c r="P251" s="57" t="n"/>
-      <c r="Q251" s="57" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="88" t="n"/>
@@ -4905,14 +4639,13 @@
       <c r="G252" s="88" t="n"/>
       <c r="H252" s="88" t="n"/>
       <c r="I252" s="88" t="n"/>
-      <c r="J252" s="112" t="n"/>
+      <c r="J252" s="88" t="n"/>
       <c r="K252" s="88" t="n"/>
       <c r="L252" s="88" t="n"/>
       <c r="M252" s="88" t="n"/>
-      <c r="N252" s="88" t="n"/>
+      <c r="N252" s="57" t="n"/>
       <c r="O252" s="57" t="n"/>
       <c r="P252" s="57" t="n"/>
-      <c r="Q252" s="57" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="88" t="n"/>
@@ -4924,14 +4657,13 @@
       <c r="G253" s="88" t="n"/>
       <c r="H253" s="88" t="n"/>
       <c r="I253" s="88" t="n"/>
-      <c r="J253" s="112" t="n"/>
+      <c r="J253" s="88" t="n"/>
       <c r="K253" s="88" t="n"/>
       <c r="L253" s="88" t="n"/>
       <c r="M253" s="88" t="n"/>
-      <c r="N253" s="88" t="n"/>
+      <c r="N253" s="57" t="n"/>
       <c r="O253" s="57" t="n"/>
       <c r="P253" s="57" t="n"/>
-      <c r="Q253" s="57" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="88" t="n"/>
@@ -4943,14 +4675,13 @@
       <c r="G254" s="88" t="n"/>
       <c r="H254" s="88" t="n"/>
       <c r="I254" s="88" t="n"/>
-      <c r="J254" s="112" t="n"/>
+      <c r="J254" s="88" t="n"/>
       <c r="K254" s="88" t="n"/>
       <c r="L254" s="88" t="n"/>
       <c r="M254" s="88" t="n"/>
-      <c r="N254" s="88" t="n"/>
+      <c r="N254" s="57" t="n"/>
       <c r="O254" s="57" t="n"/>
       <c r="P254" s="57" t="n"/>
-      <c r="Q254" s="57" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="88" t="n"/>
@@ -4962,14 +4693,13 @@
       <c r="G255" s="88" t="n"/>
       <c r="H255" s="88" t="n"/>
       <c r="I255" s="88" t="n"/>
-      <c r="J255" s="112" t="n"/>
+      <c r="J255" s="88" t="n"/>
       <c r="K255" s="88" t="n"/>
       <c r="L255" s="88" t="n"/>
       <c r="M255" s="88" t="n"/>
-      <c r="N255" s="88" t="n"/>
+      <c r="N255" s="57" t="n"/>
       <c r="O255" s="57" t="n"/>
       <c r="P255" s="57" t="n"/>
-      <c r="Q255" s="57" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="88" t="n"/>
@@ -4981,14 +4711,13 @@
       <c r="G256" s="88" t="n"/>
       <c r="H256" s="88" t="n"/>
       <c r="I256" s="88" t="n"/>
-      <c r="J256" s="112" t="n"/>
+      <c r="J256" s="88" t="n"/>
       <c r="K256" s="88" t="n"/>
       <c r="L256" s="88" t="n"/>
       <c r="M256" s="88" t="n"/>
-      <c r="N256" s="88" t="n"/>
+      <c r="N256" s="57" t="n"/>
       <c r="O256" s="57" t="n"/>
       <c r="P256" s="57" t="n"/>
-      <c r="Q256" s="57" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="9" t="n"/>
@@ -5000,14 +4729,13 @@
       <c r="G257" s="88" t="n"/>
       <c r="H257" s="88" t="n"/>
       <c r="I257" s="88" t="n"/>
-      <c r="J257" s="112" t="n"/>
+      <c r="J257" s="9" t="n"/>
       <c r="K257" s="9" t="n"/>
-      <c r="L257" s="9" t="n"/>
+      <c r="L257" s="88" t="n"/>
       <c r="M257" s="88" t="n"/>
-      <c r="N257" s="88" t="n"/>
+      <c r="N257" s="57" t="n"/>
       <c r="O257" s="57" t="n"/>
       <c r="P257" s="57" t="n"/>
-      <c r="Q257" s="57" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="9" t="n"/>
@@ -5019,14 +4747,13 @@
       <c r="G258" s="88" t="n"/>
       <c r="H258" s="88" t="n"/>
       <c r="I258" s="88" t="n"/>
-      <c r="J258" s="112" t="n"/>
+      <c r="J258" s="9" t="n"/>
       <c r="K258" s="9" t="n"/>
-      <c r="L258" s="9" t="n"/>
+      <c r="L258" s="88" t="n"/>
       <c r="M258" s="88" t="n"/>
-      <c r="N258" s="88" t="n"/>
+      <c r="N258" s="57" t="n"/>
       <c r="O258" s="57" t="n"/>
       <c r="P258" s="57" t="n"/>
-      <c r="Q258" s="57" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="9" t="n"/>
@@ -5038,14 +4765,13 @@
       <c r="G259" s="88" t="n"/>
       <c r="H259" s="88" t="n"/>
       <c r="I259" s="88" t="n"/>
-      <c r="J259" s="112" t="n"/>
+      <c r="J259" s="9" t="n"/>
       <c r="K259" s="9" t="n"/>
-      <c r="L259" s="9" t="n"/>
+      <c r="L259" s="88" t="n"/>
       <c r="M259" s="88" t="n"/>
-      <c r="N259" s="88" t="n"/>
+      <c r="N259" s="57" t="n"/>
       <c r="O259" s="57" t="n"/>
       <c r="P259" s="57" t="n"/>
-      <c r="Q259" s="57" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="9" t="n"/>
@@ -5057,14 +4783,13 @@
       <c r="G260" s="88" t="n"/>
       <c r="H260" s="88" t="n"/>
       <c r="I260" s="88" t="n"/>
-      <c r="J260" s="112" t="n"/>
+      <c r="J260" s="9" t="n"/>
       <c r="K260" s="9" t="n"/>
-      <c r="L260" s="9" t="n"/>
+      <c r="L260" s="88" t="n"/>
       <c r="M260" s="88" t="n"/>
-      <c r="N260" s="88" t="n"/>
+      <c r="N260" s="57" t="n"/>
       <c r="O260" s="57" t="n"/>
       <c r="P260" s="57" t="n"/>
-      <c r="Q260" s="57" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="9" t="n"/>
@@ -5076,14 +4801,13 @@
       <c r="G261" s="88" t="n"/>
       <c r="H261" s="88" t="n"/>
       <c r="I261" s="88" t="n"/>
-      <c r="J261" s="112" t="n"/>
+      <c r="J261" s="9" t="n"/>
       <c r="K261" s="9" t="n"/>
-      <c r="L261" s="9" t="n"/>
+      <c r="L261" s="88" t="n"/>
       <c r="M261" s="88" t="n"/>
-      <c r="N261" s="88" t="n"/>
+      <c r="N261" s="57" t="n"/>
       <c r="O261" s="57" t="n"/>
       <c r="P261" s="57" t="n"/>
-      <c r="Q261" s="57" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="9" t="n"/>
@@ -5095,14 +4819,13 @@
       <c r="G262" s="88" t="n"/>
       <c r="H262" s="88" t="n"/>
       <c r="I262" s="88" t="n"/>
-      <c r="J262" s="112" t="n"/>
+      <c r="J262" s="9" t="n"/>
       <c r="K262" s="9" t="n"/>
-      <c r="L262" s="9" t="n"/>
+      <c r="L262" s="88" t="n"/>
       <c r="M262" s="88" t="n"/>
-      <c r="N262" s="88" t="n"/>
+      <c r="N262" s="57" t="n"/>
       <c r="O262" s="57" t="n"/>
       <c r="P262" s="57" t="n"/>
-      <c r="Q262" s="57" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="9" t="n"/>
@@ -5114,14 +4837,13 @@
       <c r="G263" s="88" t="n"/>
       <c r="H263" s="88" t="n"/>
       <c r="I263" s="88" t="n"/>
-      <c r="J263" s="112" t="n"/>
+      <c r="J263" s="9" t="n"/>
       <c r="K263" s="9" t="n"/>
-      <c r="L263" s="9" t="n"/>
+      <c r="L263" s="88" t="n"/>
       <c r="M263" s="88" t="n"/>
-      <c r="N263" s="88" t="n"/>
+      <c r="N263" s="57" t="n"/>
       <c r="O263" s="57" t="n"/>
       <c r="P263" s="57" t="n"/>
-      <c r="Q263" s="57" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="9" t="n"/>
@@ -5133,14 +4855,13 @@
       <c r="G264" s="88" t="n"/>
       <c r="H264" s="88" t="n"/>
       <c r="I264" s="88" t="n"/>
-      <c r="J264" s="112" t="n"/>
+      <c r="J264" s="9" t="n"/>
       <c r="K264" s="9" t="n"/>
-      <c r="L264" s="9" t="n"/>
+      <c r="L264" s="88" t="n"/>
       <c r="M264" s="88" t="n"/>
-      <c r="N264" s="88" t="n"/>
+      <c r="N264" s="57" t="n"/>
       <c r="O264" s="57" t="n"/>
       <c r="P264" s="57" t="n"/>
-      <c r="Q264" s="57" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="9" t="n"/>
@@ -5152,14 +4873,13 @@
       <c r="G265" s="88" t="n"/>
       <c r="H265" s="88" t="n"/>
       <c r="I265" s="88" t="n"/>
-      <c r="J265" s="112" t="n"/>
+      <c r="J265" s="9" t="n"/>
       <c r="K265" s="9" t="n"/>
-      <c r="L265" s="9" t="n"/>
+      <c r="L265" s="88" t="n"/>
       <c r="M265" s="88" t="n"/>
-      <c r="N265" s="88" t="n"/>
+      <c r="N265" s="57" t="n"/>
       <c r="O265" s="57" t="n"/>
       <c r="P265" s="57" t="n"/>
-      <c r="Q265" s="57" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="9" t="n"/>
@@ -5171,35 +4891,31 @@
       <c r="G266" s="88" t="n"/>
       <c r="H266" s="88" t="n"/>
       <c r="I266" s="88" t="n"/>
-      <c r="J266" s="112" t="n"/>
+      <c r="J266" s="9" t="n"/>
       <c r="K266" s="9" t="n"/>
-      <c r="L266" s="9" t="n"/>
+      <c r="L266" s="88" t="n"/>
       <c r="M266" s="88" t="n"/>
-      <c r="N266" s="88" t="n"/>
+      <c r="N266" s="57" t="n"/>
       <c r="O266" s="57" t="n"/>
       <c r="P266" s="57" t="n"/>
-      <c r="Q266" s="57" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="15">
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="M11:N12"/>
-    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="I2:I3"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="N7:N9"/>
-    <mergeCell ref="J11:J12"/>
     <mergeCell ref="D11:D12"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="A11:A12"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="F11:F12"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L11:M12"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="C11:C12"/>
     <mergeCell ref="E11:E12"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="N2:N6"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <conditionalFormatting sqref="K13:L238">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -5212,14 +4928,11 @@
       <formula>"NA"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="J13:J238" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"AUTO"</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation sqref="I13:I238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2"</formula1>
     </dataValidation>
-    <dataValidation sqref="K13:L238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J13:K238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,NT,NA"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>